<commit_message>
docs: archive 116 passing tests for local document retrieval
</commit_message>
<xml_diff>
--- a/qa/reports/Role-AI_unit_tests_results.xlsx
+++ b/qa/reports/Role-AI_unit_tests_results.xlsx
@@ -47,7 +47,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t xml:space="preserve">요구사항별 72개 시나리오; 매개변수별 실행 수는 결과에 기록</t>
+          <t xml:space="preserve">요구사항별 84개 시나리오; 매개변수별 실행 수는 결과에 기록</t>
         </is>
       </c>
     </row>
@@ -107,7 +107,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t xml:space="preserve">00a06a66bcd85894dab689d4c3ab7b26dbe62393</t>
+          <t xml:space="preserve">1925a9f2b012d51e60e81945aa6558eff5a54d9d</t>
         </is>
       </c>
     </row>
@@ -119,7 +119,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://github.com/wjdwodhks35/Role-AI/actions/runs/38510448921</t>
+          <t xml:space="preserve">https://github.com/wjdwodhks35/Role-AI/actions/runs/38522557598</t>
         </is>
       </c>
     </row>
@@ -131,7 +131,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-10-14T04:16:11.046876+00:00</t>
+          <t xml:space="preserve">2026-10-14T06:31:15.933788+00:00</t>
         </is>
       </c>
     </row>
@@ -167,7 +167,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t xml:space="preserve">72</t>
+          <t xml:space="preserve">84</t>
         </is>
       </c>
     </row>
@@ -179,7 +179,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t xml:space="preserve">98</t>
+          <t xml:space="preserve">116</t>
         </is>
       </c>
     </row>
@@ -191,36 +191,12 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t xml:space="preserve">72</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t xml:space="preserve">초기 실행</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t xml:space="preserve">97 통과 / 1 실패: https://github.com/wjdwodhks35/Role-AI/actions/runs/38510187548</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t xml:space="preserve">경고</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t xml:space="preserve">FastAPI/Starlette TestClient 의존성 사용 중단 예정 경고 1건; 테스트 실패 없음</t>
+          <t xml:space="preserve">84</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:B17"/>
+  <autoFilter ref="A1:B15"/>
 </worksheet>
 </file>
 
@@ -362,7 +338,7 @@
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.1965</t>
+          <t xml:space="preserve">0.3715</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
@@ -434,7 +410,7 @@
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.2292</t>
+          <t xml:space="preserve">0.2438</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
@@ -506,7 +482,7 @@
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.2641</t>
+          <t xml:space="preserve">0.4451</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
@@ -578,7 +554,7 @@
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.2542</t>
+          <t xml:space="preserve">0.4394</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
@@ -650,7 +626,7 @@
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.4615</t>
+          <t xml:space="preserve">0.8113</t>
         </is>
       </c>
       <c r="N6" t="inlineStr">
@@ -722,7 +698,7 @@
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.3896</t>
+          <t xml:space="preserve">0.6196</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
@@ -794,7 +770,7 @@
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.2513</t>
+          <t xml:space="preserve">0.4403</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
@@ -866,7 +842,7 @@
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.2512</t>
+          <t xml:space="preserve">0.4354</t>
         </is>
       </c>
       <c r="N9" t="inlineStr">
@@ -938,7 +914,7 @@
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.3696</t>
+          <t xml:space="preserve">0.635</t>
         </is>
       </c>
       <c r="N10" t="inlineStr">
@@ -1010,7 +986,7 @@
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.2639</t>
+          <t xml:space="preserve">0.5252</t>
         </is>
       </c>
       <c r="N11" t="inlineStr">
@@ -1082,7 +1058,7 @@
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.26</t>
+          <t xml:space="preserve">0.4487</t>
         </is>
       </c>
       <c r="N12" t="inlineStr">
@@ -1154,7 +1130,7 @@
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.2589</t>
+          <t xml:space="preserve">0.4487</t>
         </is>
       </c>
       <c r="N13" t="inlineStr">
@@ -1226,7 +1202,7 @@
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.2363</t>
+          <t xml:space="preserve">0.2278</t>
         </is>
       </c>
       <c r="N14" t="inlineStr">
@@ -1298,7 +1274,7 @@
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t xml:space="preserve">1.2078</t>
+          <t xml:space="preserve">2.1094</t>
         </is>
       </c>
       <c r="N15" t="inlineStr">
@@ -1370,7 +1346,7 @@
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.2563</t>
+          <t xml:space="preserve">0.4379</t>
         </is>
       </c>
       <c r="N16" t="inlineStr">
@@ -1442,7 +1418,7 @@
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.4093</t>
+          <t xml:space="preserve">0.734</t>
         </is>
       </c>
       <c r="N17" t="inlineStr">
@@ -1514,7 +1490,7 @@
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.003</t>
+          <t xml:space="preserve">0.0045</t>
         </is>
       </c>
       <c r="N18" t="inlineStr">
@@ -1586,7 +1562,7 @@
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.3533</t>
+          <t xml:space="preserve">0.6191</t>
         </is>
       </c>
       <c r="N19" t="inlineStr">
@@ -1658,7 +1634,7 @@
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.0018</t>
+          <t xml:space="preserve">0.0024</t>
         </is>
       </c>
       <c r="N20" t="inlineStr">
@@ -1730,7 +1706,7 @@
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.0043</t>
+          <t xml:space="preserve">0.0062</t>
         </is>
       </c>
       <c r="N21" t="inlineStr">
@@ -1802,7 +1778,7 @@
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.0013</t>
+          <t xml:space="preserve">0.002</t>
         </is>
       </c>
       <c r="N22" t="inlineStr">
@@ -1874,7 +1850,7 @@
       </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.001</t>
+          <t xml:space="preserve">0.0015</t>
         </is>
       </c>
       <c r="N23" t="inlineStr">
@@ -1946,7 +1922,7 @@
       </c>
       <c r="M24" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.0009</t>
+          <t xml:space="preserve">0.0014</t>
         </is>
       </c>
       <c r="N24" t="inlineStr">
@@ -2018,7 +1994,7 @@
       </c>
       <c r="M25" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.2536</t>
+          <t xml:space="preserve">0.4372</t>
         </is>
       </c>
       <c r="N25" t="inlineStr">
@@ -2090,7 +2066,7 @@
       </c>
       <c r="M26" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.0002</t>
+          <t xml:space="preserve">0.0003</t>
         </is>
       </c>
       <c r="N26" t="inlineStr">
@@ -2162,7 +2138,7 @@
       </c>
       <c r="M27" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.0033</t>
+          <t xml:space="preserve">0.0045</t>
         </is>
       </c>
       <c r="N27" t="inlineStr">
@@ -2234,7 +2210,7 @@
       </c>
       <c r="M28" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.0139</t>
+          <t xml:space="preserve">0.0193</t>
         </is>
       </c>
       <c r="N28" t="inlineStr">
@@ -2306,7 +2282,7 @@
       </c>
       <c r="M29" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.0081</t>
+          <t xml:space="preserve">0.0112</t>
         </is>
       </c>
       <c r="N29" t="inlineStr">
@@ -2378,7 +2354,7 @@
       </c>
       <c r="M30" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.4884</t>
+          <t xml:space="preserve">0.8555</t>
         </is>
       </c>
       <c r="N30" t="inlineStr">
@@ -2450,7 +2426,7 @@
       </c>
       <c r="M31" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.3786</t>
+          <t xml:space="preserve">0.7014</t>
         </is>
       </c>
       <c r="N31" t="inlineStr">
@@ -2522,7 +2498,7 @@
       </c>
       <c r="M32" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.3637</t>
+          <t xml:space="preserve">0.6321</t>
         </is>
       </c>
       <c r="N32" t="inlineStr">
@@ -2594,7 +2570,7 @@
       </c>
       <c r="M33" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.3784</t>
+          <t xml:space="preserve">0.7206</t>
         </is>
       </c>
       <c r="N33" t="inlineStr">
@@ -2666,7 +2642,7 @@
       </c>
       <c r="M34" t="inlineStr">
         <is>
-          <t xml:space="preserve">2.7048</t>
+          <t xml:space="preserve">4.5065</t>
         </is>
       </c>
       <c r="N34" t="inlineStr">
@@ -2738,7 +2714,7 @@
       </c>
       <c r="M35" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.3652</t>
+          <t xml:space="preserve">0.6279</t>
         </is>
       </c>
       <c r="N35" t="inlineStr">
@@ -2810,7 +2786,7 @@
       </c>
       <c r="M36" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.4767</t>
+          <t xml:space="preserve">0.8287</t>
         </is>
       </c>
       <c r="N36" t="inlineStr">
@@ -2882,7 +2858,7 @@
       </c>
       <c r="M37" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.3666</t>
+          <t xml:space="preserve">0.6272</t>
         </is>
       </c>
       <c r="N37" t="inlineStr">
@@ -2954,7 +2930,7 @@
       </c>
       <c r="M38" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.5594</t>
+          <t xml:space="preserve">0.6547</t>
         </is>
       </c>
       <c r="N38" t="inlineStr">
@@ -3026,7 +3002,7 @@
       </c>
       <c r="M39" t="inlineStr">
         <is>
-          <t xml:space="preserve">1.4989</t>
+          <t xml:space="preserve">2.6926</t>
         </is>
       </c>
       <c r="N39" t="inlineStr">
@@ -3098,7 +3074,7 @@
       </c>
       <c r="M40" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.3778</t>
+          <t xml:space="preserve">0.6358</t>
         </is>
       </c>
       <c r="N40" t="inlineStr">
@@ -3170,7 +3146,7 @@
       </c>
       <c r="M41" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.3632</t>
+          <t xml:space="preserve">0.6305</t>
         </is>
       </c>
       <c r="N41" t="inlineStr">
@@ -3242,7 +3218,7 @@
       </c>
       <c r="M42" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.3621</t>
+          <t xml:space="preserve">0.628</t>
         </is>
       </c>
       <c r="N42" t="inlineStr">
@@ -3314,7 +3290,7 @@
       </c>
       <c r="M43" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.3704</t>
+          <t xml:space="preserve">0.6303</t>
         </is>
       </c>
       <c r="N43" t="inlineStr">
@@ -3386,7 +3362,7 @@
       </c>
       <c r="M44" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.2629</t>
+          <t xml:space="preserve">0.4457</t>
         </is>
       </c>
       <c r="N44" t="inlineStr">
@@ -3458,7 +3434,7 @@
       </c>
       <c r="M45" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.3997</t>
+          <t xml:space="preserve">0.4586</t>
         </is>
       </c>
       <c r="N45" t="inlineStr">
@@ -3530,7 +3506,7 @@
       </c>
       <c r="M46" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.2495</t>
+          <t xml:space="preserve">0.4435</t>
         </is>
       </c>
       <c r="N46" t="inlineStr">
@@ -3602,7 +3578,7 @@
       </c>
       <c r="M47" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.3615</t>
+          <t xml:space="preserve">0.7317</t>
         </is>
       </c>
       <c r="N47" t="inlineStr">
@@ -3674,7 +3650,7 @@
       </c>
       <c r="M48" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.273</t>
+          <t xml:space="preserve">0.4672</t>
         </is>
       </c>
       <c r="N48" t="inlineStr">
@@ -3746,7 +3722,7 @@
       </c>
       <c r="M49" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.2518</t>
+          <t xml:space="preserve">0.4499</t>
         </is>
       </c>
       <c r="N49" t="inlineStr">
@@ -3818,7 +3794,7 @@
       </c>
       <c r="M50" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.4926</t>
+          <t xml:space="preserve">0.8687</t>
         </is>
       </c>
       <c r="N50" t="inlineStr">
@@ -3890,7 +3866,7 @@
       </c>
       <c r="M51" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.2752</t>
+          <t xml:space="preserve">0.4672</t>
         </is>
       </c>
       <c r="N51" t="inlineStr">
@@ -3962,7 +3938,7 @@
       </c>
       <c r="M52" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.2913</t>
+          <t xml:space="preserve">0.4792</t>
         </is>
       </c>
       <c r="N52" t="inlineStr">
@@ -4034,7 +4010,7 @@
       </c>
       <c r="M53" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.4167</t>
+          <t xml:space="preserve">0.4569</t>
         </is>
       </c>
       <c r="N53" t="inlineStr">
@@ -4106,7 +4082,7 @@
       </c>
       <c r="M54" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.258</t>
+          <t xml:space="preserve">0.5366</t>
         </is>
       </c>
       <c r="N54" t="inlineStr">
@@ -4178,7 +4154,7 @@
       </c>
       <c r="M55" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.277</t>
+          <t xml:space="preserve">0.4708</t>
         </is>
       </c>
       <c r="N55" t="inlineStr">
@@ -4250,7 +4226,7 @@
       </c>
       <c r="M56" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.002</t>
+          <t xml:space="preserve">0.0027</t>
         </is>
       </c>
       <c r="N56" t="inlineStr">
@@ -4322,7 +4298,7 @@
       </c>
       <c r="M57" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.002</t>
+          <t xml:space="preserve">0.0031</t>
         </is>
       </c>
       <c r="N57" t="inlineStr">
@@ -4394,7 +4370,7 @@
       </c>
       <c r="M58" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.0018</t>
+          <t xml:space="preserve">0.0026</t>
         </is>
       </c>
       <c r="N58" t="inlineStr">
@@ -4466,7 +4442,7 @@
       </c>
       <c r="M59" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.0014</t>
+          <t xml:space="preserve">0.002</t>
         </is>
       </c>
       <c r="N59" t="inlineStr">
@@ -4538,7 +4514,7 @@
       </c>
       <c r="M60" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.374</t>
+          <t xml:space="preserve">0.6401</t>
         </is>
       </c>
       <c r="N60" t="inlineStr">
@@ -4610,7 +4586,7 @@
       </c>
       <c r="M61" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.0004</t>
+          <t xml:space="preserve">0.0006</t>
         </is>
       </c>
       <c r="N61" t="inlineStr">
@@ -4682,7 +4658,7 @@
       </c>
       <c r="M62" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.3549</t>
+          <t xml:space="preserve">0.6215</t>
         </is>
       </c>
       <c r="N62" t="inlineStr">
@@ -4754,7 +4730,7 @@
       </c>
       <c r="M63" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.3981</t>
+          <t xml:space="preserve">0.7175</t>
         </is>
       </c>
       <c r="N63" t="inlineStr">
@@ -4826,7 +4802,7 @@
       </c>
       <c r="M64" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.4324</t>
+          <t xml:space="preserve">0.6535</t>
         </is>
       </c>
       <c r="N64" t="inlineStr">
@@ -4898,7 +4874,7 @@
       </c>
       <c r="M65" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.3886</t>
+          <t xml:space="preserve">0.6617</t>
         </is>
       </c>
       <c r="N65" t="inlineStr">
@@ -4970,7 +4946,7 @@
       </c>
       <c r="M66" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.7657</t>
+          <t xml:space="preserve">0.6855</t>
         </is>
       </c>
       <c r="N66" t="inlineStr">
@@ -5042,7 +5018,7 @@
       </c>
       <c r="M67" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.5438</t>
+          <t xml:space="preserve">0.7673</t>
         </is>
       </c>
       <c r="N67" t="inlineStr">
@@ -5114,7 +5090,7 @@
       </c>
       <c r="M68" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.4304</t>
+          <t xml:space="preserve">0.6775</t>
         </is>
       </c>
       <c r="N68" t="inlineStr">
@@ -5186,7 +5162,7 @@
       </c>
       <c r="M69" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.7967</t>
+          <t xml:space="preserve">1.3408</t>
         </is>
       </c>
       <c r="N69" t="inlineStr">
@@ -5258,7 +5234,7 @@
       </c>
       <c r="M70" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.5036</t>
+          <t xml:space="preserve">0.6845</t>
         </is>
       </c>
       <c r="N70" t="inlineStr">
@@ -5330,7 +5306,7 @@
       </c>
       <c r="M71" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.486</t>
+          <t xml:space="preserve">0.8223</t>
         </is>
       </c>
       <c r="N71" t="inlineStr">
@@ -5402,7 +5378,7 @@
       </c>
       <c r="M72" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.3996</t>
+          <t xml:space="preserve">0.6807</t>
         </is>
       </c>
       <c r="N72" t="inlineStr">
@@ -5474,7 +5450,7 @@
       </c>
       <c r="M73" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.3553</t>
+          <t xml:space="preserve">0.6253</t>
         </is>
       </c>
       <c r="N73" t="inlineStr">
@@ -5483,8 +5459,872 @@
         </is>
       </c>
     </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t xml:space="preserve">73</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t xml:space="preserve">UT-073</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t xml:space="preserve">REQ-DOCUMENT-RAG</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t xml:space="preserve">documents</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t xml:space="preserve">API·단위/흐름</t>
+        </is>
+      </c>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t xml:space="preserve">문서 업로드·내보내기·중복 제거</t>
+        </is>
+      </c>
+      <c r="G74" t="inlineStr">
+        <is>
+          <t xml:space="preserve">임시 SQLite·테스트 계정·Mock 모델; 유료 API·GPU 불필요</t>
+        </is>
+      </c>
+      <c r="H74" t="inlineStr">
+        <is>
+          <t xml:space="preserve">같은 내용의 파일명을 변경해 재등록하고 다른 프로젝트 등록</t>
+        </is>
+      </c>
+      <c r="I74" t="inlineStr">
+        <is>
+          <t xml:space="preserve">동일 범위는 동일 ID, 프로젝트별 분리, 원문 내보내기 일치</t>
+        </is>
+      </c>
+      <c r="J74" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tests/test_documents.py::test_document_roundtrip_dedup_and_project</t>
+        </is>
+      </c>
+      <c r="K74" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PASS</t>
+        </is>
+      </c>
+      <c r="L74" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1</t>
+        </is>
+      </c>
+      <c r="M74" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0.5825</t>
+        </is>
+      </c>
+      <c r="N74" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t xml:space="preserve">74</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t xml:space="preserve">UT-074</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t xml:space="preserve">REQ-DOCUMENT-RAG</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t xml:space="preserve">documents</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t xml:space="preserve">API·단위/흐름</t>
+        </is>
+      </c>
+      <c r="F75" t="inlineStr">
+        <is>
+          <t xml:space="preserve">문서 입력·경로·바이너리 제한</t>
+        </is>
+      </c>
+      <c r="G75" t="inlineStr">
+        <is>
+          <t xml:space="preserve">임시 SQLite·테스트 계정·Mock 모델; 유료 API·GPU 불필요</t>
+        </is>
+      </c>
+      <c r="H75" t="inlineStr">
+        <is>
+          <t xml:space="preserve">잘못된 경로/확장자/빈 내용/제어문자/16,001자 입력</t>
+        </is>
+      </c>
+      <c r="I75" t="inlineStr">
+        <is>
+          <t xml:space="preserve">모두 422, 데이터 미저장</t>
+        </is>
+      </c>
+      <c r="J75" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tests/test_documents.py::test_document_validation</t>
+        </is>
+      </c>
+      <c r="K75" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PASS</t>
+        </is>
+      </c>
+      <c r="L75" t="inlineStr">
+        <is>
+          <t xml:space="preserve">7</t>
+        </is>
+      </c>
+      <c r="M75" t="inlineStr">
+        <is>
+          <t xml:space="preserve">3.0974</t>
+        </is>
+      </c>
+      <c r="N75" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t xml:space="preserve">75</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t xml:space="preserve">UT-075</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t xml:space="preserve">REQ-DOCUMENT-RAG</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t xml:space="preserve">documents</t>
+        </is>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t xml:space="preserve">API·단위/흐름</t>
+        </is>
+      </c>
+      <c r="F76" t="inlineStr">
+        <is>
+          <t xml:space="preserve">문서 인증·CSRF</t>
+        </is>
+      </c>
+      <c r="G76" t="inlineStr">
+        <is>
+          <t xml:space="preserve">임시 SQLite·테스트 계정·Mock 모델; 유료 API·GPU 불필요</t>
+        </is>
+      </c>
+      <c r="H76" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CSRF 없이 저장, 로그인 없이 목록/저장</t>
+        </is>
+      </c>
+      <c r="I76" t="inlineStr">
+        <is>
+          <t xml:space="preserve">403/401</t>
+        </is>
+      </c>
+      <c r="J76" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tests/test_documents.py::test_document_auth_and_csrf</t>
+        </is>
+      </c>
+      <c r="K76" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PASS</t>
+        </is>
+      </c>
+      <c r="L76" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1</t>
+        </is>
+      </c>
+      <c r="M76" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0.4356</t>
+        </is>
+      </c>
+      <c r="N76" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t xml:space="preserve">76</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t xml:space="preserve">UT-076</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t xml:space="preserve">REQ-DOCUMENT-RAG</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t xml:space="preserve">documents</t>
+        </is>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t xml:space="preserve">API·단위/흐름</t>
+        </is>
+      </c>
+      <c r="F77" t="inlineStr">
+        <is>
+          <t xml:space="preserve">문서 사용자 격리</t>
+        </is>
+      </c>
+      <c r="G77" t="inlineStr">
+        <is>
+          <t xml:space="preserve">임시 SQLite·테스트 계정·Mock 모델; 유료 API·GPU 불필요</t>
+        </is>
+      </c>
+      <c r="H77" t="inlineStr">
+        <is>
+          <t xml:space="preserve">다른 계정으로 검색/조회/다운로드/삭제/대화 참조</t>
+        </is>
+      </c>
+      <c r="I77" t="inlineStr">
+        <is>
+          <t xml:space="preserve">다른 사용자 데이터 미노출, 직접 ID 접근 404</t>
+        </is>
+      </c>
+      <c r="J77" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tests/test_documents.py::test_document_user_isolation</t>
+        </is>
+      </c>
+      <c r="K77" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PASS</t>
+        </is>
+      </c>
+      <c r="L77" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1</t>
+        </is>
+      </c>
+      <c r="M77" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0.79</t>
+        </is>
+      </c>
+      <c r="N77" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t xml:space="preserve">77</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t xml:space="preserve">UT-077</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t xml:space="preserve">REQ-DOCUMENT-RAG</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t xml:space="preserve">documents</t>
+        </is>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t xml:space="preserve">API·단위/흐름</t>
+        </is>
+      </c>
+      <c r="F78" t="inlineStr">
+        <is>
+          <t xml:space="preserve">문서 프로젝트 검색·무근거·입력 제한</t>
+        </is>
+      </c>
+      <c r="G78" t="inlineStr">
+        <is>
+          <t xml:space="preserve">임시 SQLite·테스트 계정·Mock 모델; 유료 API·GPU 불필요</t>
+        </is>
+      </c>
+      <c r="H78" t="inlineStr">
+        <is>
+          <t xml:space="preserve">공통/프로젝트별 검색, 없는 키워드, 긴 검색어</t>
+        </is>
+      </c>
+      <c r="I78" t="inlineStr">
+        <is>
+          <t xml:space="preserve">범위 내 출처만 반환, 무근거 빈 목록, 길이초과422</t>
+        </is>
+      </c>
+      <c r="J78" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tests/test_documents.py::test_document_search_scope_and_boundaries</t>
+        </is>
+      </c>
+      <c r="K78" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PASS</t>
+        </is>
+      </c>
+      <c r="L78" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1</t>
+        </is>
+      </c>
+      <c r="M78" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0.4559</t>
+        </is>
+      </c>
+      <c r="N78" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t xml:space="preserve">78</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t xml:space="preserve">UT-078</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t xml:space="preserve">REQ-DOCUMENT-RAG</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t xml:space="preserve">documents</t>
+        </is>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t xml:space="preserve">API·단위/흐름</t>
+        </is>
+      </c>
+      <c r="F79" t="inlineStr">
+        <is>
+          <t xml:space="preserve">로컬 문서 대화·출처 이력</t>
+        </is>
+      </c>
+      <c r="G79" t="inlineStr">
+        <is>
+          <t xml:space="preserve">임시 SQLite·테스트 계정·Mock 모델; 유료 API·GPU 불필요</t>
+        </is>
+      </c>
+      <c r="H79" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ollama Mock 캡처, 명령이 포함된 문서 참조</t>
+        </is>
+      </c>
+      <c r="I79" t="inlineStr">
+        <is>
+          <t xml:space="preserve">비신뢰 데이터 구분, 출처 이력 저장, 도구없음, 기억 자동저장없음</t>
+        </is>
+      </c>
+      <c r="J79" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tests/test_documents.py::test_document_chat_prompt_and_history</t>
+        </is>
+      </c>
+      <c r="K79" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PASS</t>
+        </is>
+      </c>
+      <c r="L79" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1</t>
+        </is>
+      </c>
+      <c r="M79" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0.4635</t>
+        </is>
+      </c>
+      <c r="N79" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t xml:space="preserve">79</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t xml:space="preserve">UT-079</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t xml:space="preserve">REQ-DOCUMENT-RAG</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t xml:space="preserve">documents</t>
+        </is>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t xml:space="preserve">API·단위/흐름</t>
+        </is>
+      </c>
+      <c r="F80" t="inlineStr">
+        <is>
+          <t xml:space="preserve">문서 대화 명시적 선택</t>
+        </is>
+      </c>
+      <c r="G80" t="inlineStr">
+        <is>
+          <t xml:space="preserve">임시 SQLite·테스트 계정·Mock 모델; 유료 API·GPU 불필요</t>
+        </is>
+      </c>
+      <c r="H80" t="inlineStr">
+        <is>
+          <t xml:space="preserve">미선택/일치하지 않는 문서와 대화</t>
+        </is>
+      </c>
+      <c r="I80" t="inlineStr">
+        <is>
+          <t xml:space="preserve">참고자료 자동 전송없음, 검색근거 빈 목록</t>
+        </is>
+      </c>
+      <c r="J80" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tests/test_documents.py::test_document_chat_opt_in_and_no_match</t>
+        </is>
+      </c>
+      <c r="K80" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PASS</t>
+        </is>
+      </c>
+      <c r="L80" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1</t>
+        </is>
+      </c>
+      <c r="M80" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0.4612</t>
+        </is>
+      </c>
+      <c r="N80" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t xml:space="preserve">80</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t xml:space="preserve">UT-080</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t xml:space="preserve">REQ-DOCUMENT-RAG</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t xml:space="preserve">documents</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t xml:space="preserve">API·단위/흐름</t>
+        </is>
+      </c>
+      <c r="F81" t="inlineStr">
+        <is>
+          <t xml:space="preserve">유료/별도 엔진·프로젝트 차단</t>
+        </is>
+      </c>
+      <c r="G81" t="inlineStr">
+        <is>
+          <t xml:space="preserve">임시 SQLite·테스트 계정·Mock 모델; 유료 API·GPU 불필요</t>
+        </is>
+      </c>
+      <c r="H81" t="inlineStr">
+        <is>
+          <t xml:space="preserve">OpenAI/OpenClaw/vLLM 또는 다른 프로젝트 문서 대화</t>
+        </is>
+      </c>
+      <c r="I81" t="inlineStr">
+        <is>
+          <t xml:space="preserve">403/404, 메시지 미저장</t>
+        </is>
+      </c>
+      <c r="J81" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tests/test_documents.py::test_document_chat_blocks_paid_gateway_and_wrong_project</t>
+        </is>
+      </c>
+      <c r="K81" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PASS</t>
+        </is>
+      </c>
+      <c r="L81" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1</t>
+        </is>
+      </c>
+      <c r="M81" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0.4661</t>
+        </is>
+      </c>
+      <c r="N81" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t xml:space="preserve">81</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t xml:space="preserve">UT-081</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t xml:space="preserve">REQ-DOCUMENT-RAG</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t xml:space="preserve">documents</t>
+        </is>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t xml:space="preserve">API·단위/흐름</t>
+        </is>
+      </c>
+      <c r="F82" t="inlineStr">
+        <is>
+          <t xml:space="preserve">문서 문맥·선택 수 제한</t>
+        </is>
+      </c>
+      <c r="G82" t="inlineStr">
+        <is>
+          <t xml:space="preserve">임시 SQLite·테스트 계정·Mock 모델; 유료 API·GPU 불필요</t>
+        </is>
+      </c>
+      <c r="H82" t="inlineStr">
+        <is>
+          <t xml:space="preserve">긴 문서의 여러 검색결과, 6개 선택</t>
+        </is>
+      </c>
+      <c r="I82" t="inlineStr">
+        <is>
+          <t xml:space="preserve">상위5개/JSON4500자 이하, 6개선택422</t>
+        </is>
+      </c>
+      <c r="J82" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tests/test_documents.py::test_document_context_limits_and_selection</t>
+        </is>
+      </c>
+      <c r="K82" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PASS</t>
+        </is>
+      </c>
+      <c r="L82" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1</t>
+        </is>
+      </c>
+      <c r="M82" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0.4547</t>
+        </is>
+      </c>
+      <c r="N82" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t xml:space="preserve">82</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t xml:space="preserve">UT-082</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t xml:space="preserve">REQ-DOCUMENT-RAG</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t xml:space="preserve">documents</t>
+        </is>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t xml:space="preserve">API·단위/흐름</t>
+        </is>
+      </c>
+      <c r="F83" t="inlineStr">
+        <is>
+          <t xml:space="preserve">문서 보관 한도·삭제 회수</t>
+        </is>
+      </c>
+      <c r="G83" t="inlineStr">
+        <is>
+          <t xml:space="preserve">임시 SQLite·테스트 계정·Mock 모델; 유료 API·GPU 불필요</t>
+        </is>
+      </c>
+      <c r="H83" t="inlineStr">
+        <is>
+          <t xml:space="preserve">32개 저장 후 추가/중복/삭제/재등록</t>
+        </is>
+      </c>
+      <c r="I83" t="inlineStr">
+        <is>
+          <t xml:space="preserve">추가409, 중복 허용, 발췌삭제 및 용량 회수</t>
+        </is>
+      </c>
+      <c r="J83" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tests/test_documents.py::test_document_quota_and_cleanup</t>
+        </is>
+      </c>
+      <c r="K83" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PASS</t>
+        </is>
+      </c>
+      <c r="L83" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1</t>
+        </is>
+      </c>
+      <c r="M83" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0.5791</t>
+        </is>
+      </c>
+      <c r="N83" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t xml:space="preserve">83</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t xml:space="preserve">UT-083</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t xml:space="preserve">REQ-DOCUMENT-RAG</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t xml:space="preserve">documents</t>
+        </is>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t xml:space="preserve">API·단위/흐름</t>
+        </is>
+      </c>
+      <c r="F84" t="inlineStr">
+        <is>
+          <t xml:space="preserve">문서 동시 중복 저장</t>
+        </is>
+      </c>
+      <c r="G84" t="inlineStr">
+        <is>
+          <t xml:space="preserve">임시 SQLite·테스트 계정·Mock 모델; 유료 API·GPU 불필요</t>
+        </is>
+      </c>
+      <c r="H84" t="inlineStr">
+        <is>
+          <t xml:space="preserve">8개 동일 문서 병렬 등록</t>
+        </is>
+      </c>
+      <c r="I84" t="inlineStr">
+        <is>
+          <t xml:space="preserve">저장1개 및 동일ID</t>
+        </is>
+      </c>
+      <c r="J84" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tests/test_documents.py::test_document_concurrent_duplicate</t>
+        </is>
+      </c>
+      <c r="K84" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PASS</t>
+        </is>
+      </c>
+      <c r="L84" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1</t>
+        </is>
+      </c>
+      <c r="M84" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0.4796</t>
+        </is>
+      </c>
+      <c r="N84" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t xml:space="preserve">84</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t xml:space="preserve">UT-084</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t xml:space="preserve">REQ-DOCUMENT-RAG</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t xml:space="preserve">documents</t>
+        </is>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t xml:space="preserve">API·단위/흐름</t>
+        </is>
+      </c>
+      <c r="F85" t="inlineStr">
+        <is>
+          <t xml:space="preserve">문서 삭제 후 이력·검색</t>
+        </is>
+      </c>
+      <c r="G85" t="inlineStr">
+        <is>
+          <t xml:space="preserve">임시 SQLite·테스트 계정·Mock 모델; 유료 API·GPU 불필요</t>
+        </is>
+      </c>
+      <c r="H85" t="inlineStr">
+        <is>
+          <t xml:space="preserve">대화 후 원문 삭제, 검색 및 대화 재조회</t>
+        </is>
+      </c>
+      <c r="I85" t="inlineStr">
+        <is>
+          <t xml:space="preserve">발췌검색없음, 식별자 이력 유지, 원문404</t>
+        </is>
+      </c>
+      <c r="J85" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tests/test_documents.py::test_document_deleted_source_history</t>
+        </is>
+      </c>
+      <c r="K85" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PASS</t>
+        </is>
+      </c>
+      <c r="L85" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1</t>
+        </is>
+      </c>
+      <c r="M85" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0.6074</t>
+        </is>
+      </c>
+      <c r="N85" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:N73"/>
+  <autoFilter ref="A1:N85"/>
 </worksheet>
 </file>
 
@@ -5562,17 +6402,17 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t xml:space="preserve">의미검색·문서RAG·자동 보존정책</t>
+          <t xml:space="preserve">의미검색·PDF/DOCX·자동 보존정책</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t xml:space="preserve">현재 키워드 검색만 제공</t>
+          <t xml:space="preserve">텍스트/Markdown 키워드 문서 RAG는 신규 구현; 의미 검색 등 후속</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t xml:space="preserve">미구현</t>
+          <t xml:space="preserve">부분 구현</t>
         </is>
       </c>
     </row>
@@ -5712,8 +6552,25 @@
         </is>
       </c>
     </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">REQ-DOCUMENT-RAG 문서 보관·검색·출처·로컬 대화</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">txt/md 및 키워드 RAG, 유료 호출 차단</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">자동 검증 대상</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:C13"/>
+  <autoFilter ref="A1:C14"/>
 </worksheet>
 </file>
 
@@ -5910,7 +6767,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t xml:space="preserve">PASS / https://github.com/wjdwodhks35/Role-AI/actions/runs/38510448921</t>
+          <t xml:space="preserve">PASS / https://github.com/wjdwodhks35/Role-AI/actions/runs/38522557598</t>
         </is>
       </c>
     </row>
@@ -5937,7 +6794,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t xml:space="preserve">PASS / https://github.com/wjdwodhks35/Role-AI/actions/runs/38510448921</t>
+          <t xml:space="preserve">PASS / https://github.com/wjdwodhks35/Role-AI/actions/runs/38522557598</t>
         </is>
       </c>
     </row>
@@ -7632,7 +8489,313 @@
         </is>
       </c>
     </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t xml:space="preserve">99</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tests/test_documents.py::test_document_roundtrip_dedup_and_project</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t xml:space="preserve">100</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tests/test_documents.py::test_document_validation[values0]</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t xml:space="preserve">101</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tests/test_documents.py::test_document_validation[values1]</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t xml:space="preserve">102</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tests/test_documents.py::test_document_validation[values2]</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t xml:space="preserve">103</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tests/test_documents.py::test_document_validation[values3]</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t xml:space="preserve">104</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tests/test_documents.py::test_document_validation[values4]</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t xml:space="preserve">105</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tests/test_documents.py::test_document_validation[values5]</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t xml:space="preserve">106</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tests/test_documents.py::test_document_validation[values6]</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t xml:space="preserve">107</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tests/test_documents.py::test_document_auth_and_csrf</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t xml:space="preserve">108</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tests/test_documents.py::test_document_user_isolation</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t xml:space="preserve">109</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tests/test_documents.py::test_document_search_scope_and_boundaries</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t xml:space="preserve">110</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tests/test_documents.py::test_document_chat_prompt_and_history</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t xml:space="preserve">111</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tests/test_documents.py::test_document_chat_opt_in_and_no_match</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t xml:space="preserve">112</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tests/test_documents.py::test_document_chat_blocks_paid_gateway_and_wrong_project</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t xml:space="preserve">113</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tests/test_documents.py::test_document_context_limits_and_selection</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t xml:space="preserve">114</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tests/test_documents.py::test_document_quota_and_cleanup</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t xml:space="preserve">115</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tests/test_documents.py::test_document_concurrent_duplicate</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t xml:space="preserve">116</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tests/test_documents.py::test_document_deleted_source_history</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PASS</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:C99"/>
+  <autoFilter ref="A1:C117"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
docs: record 141 passing tests including Docker host retrieval
</commit_message>
<xml_diff>
--- a/qa/reports/Role-AI_unit_tests_results.xlsx
+++ b/qa/reports/Role-AI_unit_tests_results.xlsx
@@ -107,7 +107,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t xml:space="preserve">e218185b57a426cc947970b959ce021a851e7caa</t>
+          <t xml:space="preserve">1ff9e4fd4e7b9d151c2cb2297ecb03b5a9fa6358</t>
         </is>
       </c>
     </row>
@@ -119,7 +119,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://github.com/wjdwodhks35/Role-AI/actions/runs/38525399524</t>
+          <t xml:space="preserve">https://github.com/wjdwodhks35/Role-AI/actions/runs/38526015394</t>
         </is>
       </c>
     </row>
@@ -131,7 +131,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-10-14T07:00:04.241361+00:00</t>
+          <t xml:space="preserve">2026-10-14T07:06:01.142455+00:00</t>
         </is>
       </c>
     </row>
@@ -179,7 +179,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t xml:space="preserve">138</t>
+          <t xml:space="preserve">141</t>
         </is>
       </c>
     </row>
@@ -338,7 +338,7 @@
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.2662</t>
+          <t xml:space="preserve">0.3139</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
@@ -410,7 +410,7 @@
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.7142</t>
+          <t xml:space="preserve">0.2425</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
@@ -482,7 +482,7 @@
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t xml:space="preserve">1.804</t>
+          <t xml:space="preserve">0.4355</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
@@ -554,7 +554,7 @@
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.3243</t>
+          <t xml:space="preserve">0.4273</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
@@ -626,7 +626,7 @@
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.6022</t>
+          <t xml:space="preserve">0.7785</t>
         </is>
       </c>
       <c r="N6" t="inlineStr">
@@ -698,7 +698,7 @@
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.5234</t>
+          <t xml:space="preserve">0.5936</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
@@ -770,7 +770,7 @@
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.4018</t>
+          <t xml:space="preserve">0.482</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
@@ -842,7 +842,7 @@
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.3619</t>
+          <t xml:space="preserve">0.4223</t>
         </is>
       </c>
       <c r="N9" t="inlineStr">
@@ -914,7 +914,7 @@
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.4722</t>
+          <t xml:space="preserve">0.6168</t>
         </is>
       </c>
       <c r="N10" t="inlineStr">
@@ -986,7 +986,7 @@
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.3843</t>
+          <t xml:space="preserve">0.4402</t>
         </is>
       </c>
       <c r="N11" t="inlineStr">
@@ -1058,7 +1058,7 @@
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.3948</t>
+          <t xml:space="preserve">0.4405</t>
         </is>
       </c>
       <c r="N12" t="inlineStr">
@@ -1130,7 +1130,7 @@
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.3416</t>
+          <t xml:space="preserve">0.4417</t>
         </is>
       </c>
       <c r="N13" t="inlineStr">
@@ -1202,7 +1202,7 @@
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.1712</t>
+          <t xml:space="preserve">0.2417</t>
         </is>
       </c>
       <c r="N14" t="inlineStr">
@@ -1274,7 +1274,7 @@
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t xml:space="preserve">1.5561</t>
+          <t xml:space="preserve">2.26</t>
         </is>
       </c>
       <c r="N15" t="inlineStr">
@@ -1346,7 +1346,7 @@
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.6395</t>
+          <t xml:space="preserve">0.4309</t>
         </is>
       </c>
       <c r="N16" t="inlineStr">
@@ -1418,7 +1418,7 @@
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.5243</t>
+          <t xml:space="preserve">0.6908</t>
         </is>
       </c>
       <c r="N17" t="inlineStr">
@@ -1490,7 +1490,7 @@
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.0041</t>
+          <t xml:space="preserve">0.0054</t>
         </is>
       </c>
       <c r="N18" t="inlineStr">
@@ -1562,7 +1562,7 @@
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.5119</t>
+          <t xml:space="preserve">0.632</t>
         </is>
       </c>
       <c r="N19" t="inlineStr">
@@ -1634,7 +1634,7 @@
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.0021</t>
+          <t xml:space="preserve">0.0027</t>
         </is>
       </c>
       <c r="N20" t="inlineStr">
@@ -1706,7 +1706,7 @@
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.0054</t>
+          <t xml:space="preserve">0.007</t>
         </is>
       </c>
       <c r="N21" t="inlineStr">
@@ -1778,7 +1778,7 @@
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.0966</t>
+          <t xml:space="preserve">0.0684</t>
         </is>
       </c>
       <c r="N22" t="inlineStr">
@@ -1850,7 +1850,7 @@
       </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.0016</t>
+          <t xml:space="preserve">0.002</t>
         </is>
       </c>
       <c r="N23" t="inlineStr">
@@ -1922,7 +1922,7 @@
       </c>
       <c r="M24" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.0013</t>
+          <t xml:space="preserve">0.0017</t>
         </is>
       </c>
       <c r="N24" t="inlineStr">
@@ -1994,7 +1994,7 @@
       </c>
       <c r="M25" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.3285</t>
+          <t xml:space="preserve">0.4245</t>
         </is>
       </c>
       <c r="N25" t="inlineStr">
@@ -2066,7 +2066,7 @@
       </c>
       <c r="M26" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.0003</t>
+          <t xml:space="preserve">0.0004</t>
         </is>
       </c>
       <c r="N26" t="inlineStr">
@@ -2138,7 +2138,7 @@
       </c>
       <c r="M27" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.004</t>
+          <t xml:space="preserve">0.0049</t>
         </is>
       </c>
       <c r="N27" t="inlineStr">
@@ -2210,7 +2210,7 @@
       </c>
       <c r="M28" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.0176</t>
+          <t xml:space="preserve">0.0226</t>
         </is>
       </c>
       <c r="N28" t="inlineStr">
@@ -2282,7 +2282,7 @@
       </c>
       <c r="M29" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.0103</t>
+          <t xml:space="preserve">0.0128</t>
         </is>
       </c>
       <c r="N29" t="inlineStr">
@@ -2354,7 +2354,7 @@
       </c>
       <c r="M30" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.921</t>
+          <t xml:space="preserve">0.8171</t>
         </is>
       </c>
       <c r="N30" t="inlineStr">
@@ -2426,7 +2426,7 @@
       </c>
       <c r="M31" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.5515</t>
+          <t xml:space="preserve">0.618</t>
         </is>
       </c>
       <c r="N31" t="inlineStr">
@@ -2498,7 +2498,7 @@
       </c>
       <c r="M32" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.5628</t>
+          <t xml:space="preserve">0.6427</t>
         </is>
       </c>
       <c r="N32" t="inlineStr">
@@ -2570,7 +2570,7 @@
       </c>
       <c r="M33" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.4881</t>
+          <t xml:space="preserve">0.6225</t>
         </is>
       </c>
       <c r="N33" t="inlineStr">
@@ -2642,7 +2642,7 @@
       </c>
       <c r="M34" t="inlineStr">
         <is>
-          <t xml:space="preserve">4.7799</t>
+          <t xml:space="preserve">4.3925</t>
         </is>
       </c>
       <c r="N34" t="inlineStr">
@@ -2714,7 +2714,7 @@
       </c>
       <c r="M35" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.5296</t>
+          <t xml:space="preserve">0.608</t>
         </is>
       </c>
       <c r="N35" t="inlineStr">
@@ -2786,7 +2786,7 @@
       </c>
       <c r="M36" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.8089</t>
+          <t xml:space="preserve">0.7998</t>
         </is>
       </c>
       <c r="N36" t="inlineStr">
@@ -2858,7 +2858,7 @@
       </c>
       <c r="M37" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.5997</t>
+          <t xml:space="preserve">0.6101</t>
         </is>
       </c>
       <c r="N37" t="inlineStr">
@@ -2930,7 +2930,7 @@
       </c>
       <c r="M38" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.5598</t>
+          <t xml:space="preserve">0.6342</t>
         </is>
       </c>
       <c r="N38" t="inlineStr">
@@ -3002,7 +3002,7 @@
       </c>
       <c r="M39" t="inlineStr">
         <is>
-          <t xml:space="preserve">3.064</t>
+          <t xml:space="preserve">2.5859</t>
         </is>
       </c>
       <c r="N39" t="inlineStr">
@@ -3074,7 +3074,7 @@
       </c>
       <c r="M40" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.5077</t>
+          <t xml:space="preserve">0.6513</t>
         </is>
       </c>
       <c r="N40" t="inlineStr">
@@ -3146,7 +3146,7 @@
       </c>
       <c r="M41" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.5</t>
+          <t xml:space="preserve">0.604</t>
         </is>
       </c>
       <c r="N41" t="inlineStr">
@@ -3218,7 +3218,7 @@
       </c>
       <c r="M42" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.5156</t>
+          <t xml:space="preserve">0.6053</t>
         </is>
       </c>
       <c r="N42" t="inlineStr">
@@ -3290,7 +3290,7 @@
       </c>
       <c r="M43" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.4692</t>
+          <t xml:space="preserve">0.6106</t>
         </is>
       </c>
       <c r="N43" t="inlineStr">
@@ -3362,7 +3362,7 @@
       </c>
       <c r="M44" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.5242</t>
+          <t xml:space="preserve">0.526</t>
         </is>
       </c>
       <c r="N44" t="inlineStr">
@@ -3434,7 +3434,7 @@
       </c>
       <c r="M45" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.4425</t>
+          <t xml:space="preserve">0.4771</t>
         </is>
       </c>
       <c r="N45" t="inlineStr">
@@ -3506,7 +3506,7 @@
       </c>
       <c r="M46" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.3415</t>
+          <t xml:space="preserve">0.435</t>
         </is>
       </c>
       <c r="N46" t="inlineStr">
@@ -3578,7 +3578,7 @@
       </c>
       <c r="M47" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.4869</t>
+          <t xml:space="preserve">0.6144</t>
         </is>
       </c>
       <c r="N47" t="inlineStr">
@@ -3650,7 +3650,7 @@
       </c>
       <c r="M48" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.3709</t>
+          <t xml:space="preserve">0.4582</t>
         </is>
       </c>
       <c r="N48" t="inlineStr">
@@ -3722,7 +3722,7 @@
       </c>
       <c r="M49" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.3379</t>
+          <t xml:space="preserve">0.4591</t>
         </is>
       </c>
       <c r="N49" t="inlineStr">
@@ -3794,7 +3794,7 @@
       </c>
       <c r="M50" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.8146</t>
+          <t xml:space="preserve">0.8646</t>
         </is>
       </c>
       <c r="N50" t="inlineStr">
@@ -3866,7 +3866,7 @@
       </c>
       <c r="M51" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.534</t>
+          <t xml:space="preserve">0.5663</t>
         </is>
       </c>
       <c r="N51" t="inlineStr">
@@ -3938,7 +3938,7 @@
       </c>
       <c r="M52" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.4321</t>
+          <t xml:space="preserve">0.4759</t>
         </is>
       </c>
       <c r="N52" t="inlineStr">
@@ -4010,7 +4010,7 @@
       </c>
       <c r="M53" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.5792</t>
+          <t xml:space="preserve">0.4598</t>
         </is>
       </c>
       <c r="N53" t="inlineStr">
@@ -4082,7 +4082,7 @@
       </c>
       <c r="M54" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.3537</t>
+          <t xml:space="preserve">0.4286</t>
         </is>
       </c>
       <c r="N54" t="inlineStr">
@@ -4154,7 +4154,7 @@
       </c>
       <c r="M55" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.523</t>
+          <t xml:space="preserve">0.466</t>
         </is>
       </c>
       <c r="N55" t="inlineStr">
@@ -4226,7 +4226,7 @@
       </c>
       <c r="M56" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.0024</t>
+          <t xml:space="preserve">0.003</t>
         </is>
       </c>
       <c r="N56" t="inlineStr">
@@ -4298,7 +4298,7 @@
       </c>
       <c r="M57" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.0027</t>
+          <t xml:space="preserve">0.0035</t>
         </is>
       </c>
       <c r="N57" t="inlineStr">
@@ -4370,7 +4370,7 @@
       </c>
       <c r="M58" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.0022</t>
+          <t xml:space="preserve">0.003</t>
         </is>
       </c>
       <c r="N58" t="inlineStr">
@@ -4442,7 +4442,7 @@
       </c>
       <c r="M59" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.0018</t>
+          <t xml:space="preserve">0.0025</t>
         </is>
       </c>
       <c r="N59" t="inlineStr">
@@ -4514,7 +4514,7 @@
       </c>
       <c r="M60" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.6121</t>
+          <t xml:space="preserve">0.6286</t>
         </is>
       </c>
       <c r="N60" t="inlineStr">
@@ -4586,7 +4586,7 @@
       </c>
       <c r="M61" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.0006</t>
+          <t xml:space="preserve">0.0007</t>
         </is>
       </c>
       <c r="N61" t="inlineStr">
@@ -4658,7 +4658,7 @@
       </c>
       <c r="M62" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.4517</t>
+          <t xml:space="preserve">0.6379</t>
         </is>
       </c>
       <c r="N62" t="inlineStr">
@@ -4730,7 +4730,7 @@
       </c>
       <c r="M63" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.5207</t>
+          <t xml:space="preserve">0.6528</t>
         </is>
       </c>
       <c r="N63" t="inlineStr">
@@ -4802,7 +4802,7 @@
       </c>
       <c r="M64" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.878</t>
+          <t xml:space="preserve">0.6351</t>
         </is>
       </c>
       <c r="N64" t="inlineStr">
@@ -4874,7 +4874,7 @@
       </c>
       <c r="M65" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.6119</t>
+          <t xml:space="preserve">0.7576</t>
         </is>
       </c>
       <c r="N65" t="inlineStr">
@@ -4946,7 +4946,7 @@
       </c>
       <c r="M66" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.8142</t>
+          <t xml:space="preserve">0.6678</t>
         </is>
       </c>
       <c r="N66" t="inlineStr">
@@ -5018,7 +5018,7 @@
       </c>
       <c r="M67" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.4863</t>
+          <t xml:space="preserve">0.6487</t>
         </is>
       </c>
       <c r="N67" t="inlineStr">
@@ -5090,7 +5090,7 @@
       </c>
       <c r="M68" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.5075</t>
+          <t xml:space="preserve">0.6802</t>
         </is>
       </c>
       <c r="N68" t="inlineStr">
@@ -5162,7 +5162,7 @@
       </c>
       <c r="M69" t="inlineStr">
         <is>
-          <t xml:space="preserve">1.0513</t>
+          <t xml:space="preserve">1.3338</t>
         </is>
       </c>
       <c r="N69" t="inlineStr">
@@ -5234,7 +5234,7 @@
       </c>
       <c r="M70" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.518</t>
+          <t xml:space="preserve">0.6644</t>
         </is>
       </c>
       <c r="N70" t="inlineStr">
@@ -5306,7 +5306,7 @@
       </c>
       <c r="M71" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.7827</t>
+          <t xml:space="preserve">0.8962</t>
         </is>
       </c>
       <c r="N71" t="inlineStr">
@@ -5378,7 +5378,7 @@
       </c>
       <c r="M72" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.537</t>
+          <t xml:space="preserve">0.6577</t>
         </is>
       </c>
       <c r="N72" t="inlineStr">
@@ -5450,7 +5450,7 @@
       </c>
       <c r="M73" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.7639</t>
+          <t xml:space="preserve">0.5968</t>
         </is>
       </c>
       <c r="N73" t="inlineStr">
@@ -5522,7 +5522,7 @@
       </c>
       <c r="M74" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.3449</t>
+          <t xml:space="preserve">0.4496</t>
         </is>
       </c>
       <c r="N74" t="inlineStr">
@@ -5594,7 +5594,7 @@
       </c>
       <c r="M75" t="inlineStr">
         <is>
-          <t xml:space="preserve">2.6091</t>
+          <t xml:space="preserve">3.1217</t>
         </is>
       </c>
       <c r="N75" t="inlineStr">
@@ -5666,7 +5666,7 @@
       </c>
       <c r="M76" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.3217</t>
+          <t xml:space="preserve">0.4239</t>
         </is>
       </c>
       <c r="N76" t="inlineStr">
@@ -5738,7 +5738,7 @@
       </c>
       <c r="M77" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.7428</t>
+          <t xml:space="preserve">0.6381</t>
         </is>
       </c>
       <c r="N77" t="inlineStr">
@@ -5810,7 +5810,7 @@
       </c>
       <c r="M78" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.7798</t>
+          <t xml:space="preserve">0.4498</t>
         </is>
       </c>
       <c r="N78" t="inlineStr">
@@ -5882,7 +5882,7 @@
       </c>
       <c r="M79" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.4421</t>
+          <t xml:space="preserve">0.457</t>
         </is>
       </c>
       <c r="N79" t="inlineStr">
@@ -5954,7 +5954,7 @@
       </c>
       <c r="M80" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.8</t>
+          <t xml:space="preserve">0.4845</t>
         </is>
       </c>
       <c r="N80" t="inlineStr">
@@ -6026,7 +6026,7 @@
       </c>
       <c r="M81" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.384</t>
+          <t xml:space="preserve">0.455</t>
         </is>
       </c>
       <c r="N81" t="inlineStr">
@@ -6098,7 +6098,7 @@
       </c>
       <c r="M82" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.7064</t>
+          <t xml:space="preserve">0.5846</t>
         </is>
       </c>
       <c r="N82" t="inlineStr">
@@ -6170,7 +6170,7 @@
       </c>
       <c r="M83" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.4977</t>
+          <t xml:space="preserve">0.5941</t>
         </is>
       </c>
       <c r="N83" t="inlineStr">
@@ -6242,7 +6242,7 @@
       </c>
       <c r="M84" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.3654</t>
+          <t xml:space="preserve">0.47</t>
         </is>
       </c>
       <c r="N84" t="inlineStr">
@@ -6314,7 +6314,7 @@
       </c>
       <c r="M85" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.3674</t>
+          <t xml:space="preserve">0.4695</t>
         </is>
       </c>
       <c r="N85" t="inlineStr">
@@ -6386,7 +6386,7 @@
       </c>
       <c r="M86" t="inlineStr">
         <is>
-          <t xml:space="preserve">1.2156</t>
+          <t xml:space="preserve">1.2381</t>
         </is>
       </c>
       <c r="N86" t="inlineStr">
@@ -6458,7 +6458,7 @@
       </c>
       <c r="M87" t="inlineStr">
         <is>
-          <t xml:space="preserve">4.0715</t>
+          <t xml:space="preserve">4.7279</t>
         </is>
       </c>
       <c r="N87" t="inlineStr">
@@ -6530,7 +6530,7 @@
       </c>
       <c r="M88" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.7038</t>
+          <t xml:space="preserve">0.8946</t>
         </is>
       </c>
       <c r="N88" t="inlineStr">
@@ -6602,7 +6602,7 @@
       </c>
       <c r="M89" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.4047</t>
+          <t xml:space="preserve">0.4454</t>
         </is>
       </c>
       <c r="N89" t="inlineStr">
@@ -6649,7 +6649,7 @@
       </c>
       <c r="H90" t="inlineStr">
         <is>
-          <t xml:space="preserve">키워드가 없는 질의, Mock 로컬 임베딩으로 유사 문서 검색</t>
+          <t xml:space="preserve">키워드가 없는 질의, Mock 로컬 임베딩으로 유사 문서 검색; localhost/127.0.0.1/IPv6/Docker host-gateway 주소 검증</t>
         </is>
       </c>
       <c r="I90" t="inlineStr">
@@ -6669,12 +6669,12 @@
       </c>
       <c r="L90" t="inlineStr">
         <is>
-          <t xml:space="preserve">1</t>
+          <t xml:space="preserve">4</t>
         </is>
       </c>
       <c r="M90" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.3387</t>
+          <t xml:space="preserve">1.7801</t>
         </is>
       </c>
       <c r="N90" t="inlineStr">
@@ -6746,7 +6746,7 @@
       </c>
       <c r="M91" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.3322</t>
+          <t xml:space="preserve">0.6096</t>
         </is>
       </c>
       <c r="N91" t="inlineStr">
@@ -6818,7 +6818,7 @@
       </c>
       <c r="M92" t="inlineStr">
         <is>
-          <t xml:space="preserve">3.4628</t>
+          <t xml:space="preserve">3.0818</t>
         </is>
       </c>
       <c r="N92" t="inlineStr">
@@ -6890,7 +6890,7 @@
       </c>
       <c r="M93" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.3373</t>
+          <t xml:space="preserve">0.4535</t>
         </is>
       </c>
       <c r="N93" t="inlineStr">
@@ -6962,7 +6962,7 @@
       </c>
       <c r="M94" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.6972</t>
+          <t xml:space="preserve">0.6146</t>
         </is>
       </c>
       <c r="N94" t="inlineStr">
@@ -7034,7 +7034,7 @@
       </c>
       <c r="M95" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.3681</t>
+          <t xml:space="preserve">0.6263</t>
         </is>
       </c>
       <c r="N95" t="inlineStr">
@@ -7106,7 +7106,7 @@
       </c>
       <c r="M96" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.365</t>
+          <t xml:space="preserve">0.451</t>
         </is>
       </c>
       <c r="N96" t="inlineStr">
@@ -7598,7 +7598,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t xml:space="preserve">PASS / https://github.com/wjdwodhks35/Role-AI/actions/runs/38525399524</t>
+          <t xml:space="preserve">PASS / https://github.com/wjdwodhks35/Role-AI/actions/runs/38526015394</t>
         </is>
       </c>
     </row>
@@ -7625,7 +7625,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t xml:space="preserve">PASS / https://github.com/wjdwodhks35/Role-AI/actions/runs/38525399524</t>
+          <t xml:space="preserve">PASS / https://github.com/wjdwodhks35/Role-AI/actions/runs/38526015394</t>
         </is>
       </c>
     </row>
@@ -9787,7 +9787,7 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t xml:space="preserve">tests/test_pdf_semantic.py::test_semantic_synonyms_without_keyword_match</t>
+          <t xml:space="preserve">tests/test_pdf_semantic.py::test_semantic_synonyms_without_keyword_match[localhost]</t>
         </is>
       </c>
       <c r="C127" t="inlineStr">
@@ -9804,7 +9804,7 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t xml:space="preserve">tests/test_pdf_semantic.py::test_semantic_disabled_and_no_hidden_fallback</t>
+          <t xml:space="preserve">tests/test_pdf_semantic.py::test_semantic_synonyms_without_keyword_match[127.0.0.1]</t>
         </is>
       </c>
       <c r="C128" t="inlineStr">
@@ -9821,7 +9821,7 @@
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t xml:space="preserve">tests/test_pdf_semantic.py::test_semantic_invalid_vectors[response0]</t>
+          <t xml:space="preserve">tests/test_pdf_semantic.py::test_semantic_synonyms_without_keyword_match[[::1]]</t>
         </is>
       </c>
       <c r="C129" t="inlineStr">
@@ -9838,7 +9838,7 @@
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t xml:space="preserve">tests/test_pdf_semantic.py::test_semantic_invalid_vectors[response1]</t>
+          <t xml:space="preserve">tests/test_pdf_semantic.py::test_semantic_synonyms_without_keyword_match[host.docker.internal]</t>
         </is>
       </c>
       <c r="C130" t="inlineStr">
@@ -9855,7 +9855,7 @@
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t xml:space="preserve">tests/test_pdf_semantic.py::test_semantic_invalid_vectors[response2]</t>
+          <t xml:space="preserve">tests/test_pdf_semantic.py::test_semantic_disabled_and_no_hidden_fallback</t>
         </is>
       </c>
       <c r="C131" t="inlineStr">
@@ -9872,7 +9872,7 @@
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t xml:space="preserve">tests/test_pdf_semantic.py::test_semantic_invalid_vectors[response3]</t>
+          <t xml:space="preserve">tests/test_pdf_semantic.py::test_semantic_invalid_vectors[response0]</t>
         </is>
       </c>
       <c r="C132" t="inlineStr">
@@ -9889,7 +9889,7 @@
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t xml:space="preserve">tests/test_pdf_semantic.py::test_semantic_invalid_vectors[response4]</t>
+          <t xml:space="preserve">tests/test_pdf_semantic.py::test_semantic_invalid_vectors[response1]</t>
         </is>
       </c>
       <c r="C133" t="inlineStr">
@@ -9906,7 +9906,7 @@
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t xml:space="preserve">tests/test_pdf_semantic.py::test_semantic_invalid_vectors[response5]</t>
+          <t xml:space="preserve">tests/test_pdf_semantic.py::test_semantic_invalid_vectors[response2]</t>
         </is>
       </c>
       <c r="C134" t="inlineStr">
@@ -9923,7 +9923,7 @@
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t xml:space="preserve">tests/test_pdf_semantic.py::test_semantic_invalid_vectors[response6]</t>
+          <t xml:space="preserve">tests/test_pdf_semantic.py::test_semantic_invalid_vectors[response3]</t>
         </is>
       </c>
       <c r="C135" t="inlineStr">
@@ -9940,7 +9940,7 @@
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t xml:space="preserve">tests/test_pdf_semantic.py::test_semantic_remote_and_cloud_models_blocked</t>
+          <t xml:space="preserve">tests/test_pdf_semantic.py::test_semantic_invalid_vectors[response4]</t>
         </is>
       </c>
       <c r="C136" t="inlineStr">
@@ -9957,7 +9957,7 @@
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t xml:space="preserve">tests/test_pdf_semantic.py::test_semantic_user_project_and_csrf_before_inference</t>
+          <t xml:space="preserve">tests/test_pdf_semantic.py::test_semantic_invalid_vectors[response5]</t>
         </is>
       </c>
       <c r="C137" t="inlineStr">
@@ -9974,7 +9974,7 @@
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t xml:space="preserve">tests/test_pdf_semantic.py::test_semantic_chat_context_history_and_paid_block</t>
+          <t xml:space="preserve">tests/test_pdf_semantic.py::test_semantic_invalid_vectors[response6]</t>
         </is>
       </c>
       <c r="C138" t="inlineStr">
@@ -9991,16 +9991,67 @@
       </c>
       <c r="B139" t="inlineStr">
         <is>
+          <t xml:space="preserve">tests/test_pdf_semantic.py::test_semantic_remote_and_cloud_models_blocked</t>
+        </is>
+      </c>
+      <c r="C139" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t xml:space="preserve">139</t>
+        </is>
+      </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tests/test_pdf_semantic.py::test_semantic_user_project_and_csrf_before_inference</t>
+        </is>
+      </c>
+      <c r="C140" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t xml:space="preserve">140</t>
+        </is>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tests/test_pdf_semantic.py::test_semantic_chat_context_history_and_paid_block</t>
+        </is>
+      </c>
+      <c r="C141" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t xml:space="preserve">141</t>
+        </is>
+      </c>
+      <c r="B142" t="inlineStr">
+        <is>
           <t xml:space="preserve">tests/test_pdf_semantic.py::test_semantic_timeout_no_history_and_gpu_lock</t>
         </is>
       </c>
-      <c r="C139" t="inlineStr">
+      <c r="C142" t="inlineStr">
         <is>
           <t xml:space="preserve">PASS</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:C139"/>
+  <autoFilter ref="A1:C142"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
docs: record 142 ordered scenarios and 211 passing executions with review scope
</commit_message>
<xml_diff>
--- a/qa/reports/Role-AI_unit_tests_results.xlsx
+++ b/qa/reports/Role-AI_unit_tests_results.xlsx
@@ -47,7 +47,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t xml:space="preserve">129개 시나리오; 매개변수별 실행 수는 결과에 기록</t>
+          <t xml:space="preserve">142개 시나리오; 매개변수별 실행 수는 결과에 기록</t>
         </is>
       </c>
     </row>
@@ -90,113 +90,101 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t xml:space="preserve">결과</t>
+          <t xml:space="preserve">commit</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t xml:space="preserve">실행 전: 결과 파일은 CI에서 별도 생성</t>
+          <t xml:space="preserve">06c068f358bed1a952e0538e2a86ccf8b34c1a51</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t xml:space="preserve">commit</t>
+          <t xml:space="preserve">run_url</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t xml:space="preserve">9c410f7a2a27be006945103bb01168fa3ab36c24</t>
+          <t xml:space="preserve">https://github.com/wjdwodhks35/Role-AI/actions/runs/38539414117</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t xml:space="preserve">run_url</t>
+          <t xml:space="preserve">utc</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://github.com/wjdwodhks35/Role-AI/actions/runs/38536591380</t>
+          <t xml:space="preserve">2026-10-14T09:04:36.807097+00:00</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t xml:space="preserve">utc</t>
+          <t xml:space="preserve">ordered</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-10-14T08:40:54.594281+00:00</t>
+          <t xml:space="preserve">true</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t xml:space="preserve">ordered</t>
+          <t xml:space="preserve">exit_code</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t xml:space="preserve">true</t>
+          <t xml:space="preserve">0</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t xml:space="preserve">exit_code</t>
+          <t xml:space="preserve">scenarios</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t xml:space="preserve">0</t>
+          <t xml:space="preserve">142</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t xml:space="preserve">scenarios</t>
+          <t xml:space="preserve">executions</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t xml:space="preserve">129</t>
+          <t xml:space="preserve">211</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t xml:space="preserve">executions</t>
+          <t xml:space="preserve">passed_scenarios</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t xml:space="preserve">189</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t xml:space="preserve">passed_scenarios</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t xml:space="preserve">129</t>
+          <t xml:space="preserve">142</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:B15"/>
+  <autoFilter ref="A1:B14"/>
 </worksheet>
 </file>
 
@@ -338,7 +326,7 @@
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.341</t>
+          <t xml:space="preserve">0.426</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
@@ -410,7 +398,7 @@
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.2924</t>
+          <t xml:space="preserve">0.2675</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
@@ -482,7 +470,7 @@
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.4541</t>
+          <t xml:space="preserve">0.4624</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
@@ -554,7 +542,7 @@
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.4434</t>
+          <t xml:space="preserve">0.4695</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
@@ -626,7 +614,7 @@
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.8011</t>
+          <t xml:space="preserve">0.8035</t>
         </is>
       </c>
       <c r="N6" t="inlineStr">
@@ -698,7 +686,7 @@
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.6142</t>
+          <t xml:space="preserve">0.6207</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
@@ -770,7 +758,7 @@
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.4404</t>
+          <t xml:space="preserve">0.4539</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
@@ -842,7 +830,7 @@
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.4416</t>
+          <t xml:space="preserve">0.5296</t>
         </is>
       </c>
       <c r="N9" t="inlineStr">
@@ -914,7 +902,7 @@
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.6336</t>
+          <t xml:space="preserve">0.6367</t>
         </is>
       </c>
       <c r="N10" t="inlineStr">
@@ -986,7 +974,7 @@
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.5346</t>
+          <t xml:space="preserve">0.4642</t>
         </is>
       </c>
       <c r="N11" t="inlineStr">
@@ -1058,7 +1046,7 @@
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.4503</t>
+          <t xml:space="preserve">0.46</t>
         </is>
       </c>
       <c r="N12" t="inlineStr">
@@ -1130,7 +1118,7 @@
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.4518</t>
+          <t xml:space="preserve">0.4627</t>
         </is>
       </c>
       <c r="N13" t="inlineStr">
@@ -1202,7 +1190,7 @@
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.2335</t>
+          <t xml:space="preserve">0.2376</t>
         </is>
       </c>
       <c r="N14" t="inlineStr">
@@ -1274,7 +1262,7 @@
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t xml:space="preserve">2.0185</t>
+          <t xml:space="preserve">2.0232</t>
         </is>
       </c>
       <c r="N15" t="inlineStr">
@@ -1346,7 +1334,7 @@
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.4548</t>
+          <t xml:space="preserve">0.5488</t>
         </is>
       </c>
       <c r="N16" t="inlineStr">
@@ -1418,7 +1406,7 @@
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.6954</t>
+          <t xml:space="preserve">0.6932</t>
         </is>
       </c>
       <c r="N17" t="inlineStr">
@@ -1562,7 +1550,7 @@
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.6076</t>
+          <t xml:space="preserve">0.6205</t>
         </is>
       </c>
       <c r="N19" t="inlineStr">
@@ -1634,7 +1622,7 @@
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.0028</t>
+          <t xml:space="preserve">0.0031</t>
         </is>
       </c>
       <c r="N20" t="inlineStr">
@@ -1706,7 +1694,7 @@
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.0074</t>
+          <t xml:space="preserve">0.0078</t>
         </is>
       </c>
       <c r="N21" t="inlineStr">
@@ -1778,7 +1766,7 @@
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.0023</t>
+          <t xml:space="preserve">0.0026</t>
         </is>
       </c>
       <c r="N22" t="inlineStr">
@@ -1994,7 +1982,7 @@
       </c>
       <c r="M25" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.5245</t>
+          <t xml:space="preserve">0.4451</t>
         </is>
       </c>
       <c r="N25" t="inlineStr">
@@ -2210,7 +2198,7 @@
       </c>
       <c r="M28" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.0231</t>
+          <t xml:space="preserve">0.0242</t>
         </is>
       </c>
       <c r="N28" t="inlineStr">
@@ -2282,7 +2270,7 @@
       </c>
       <c r="M29" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.0134</t>
+          <t xml:space="preserve">0.0133</t>
         </is>
       </c>
       <c r="N29" t="inlineStr">
@@ -2354,7 +2342,7 @@
       </c>
       <c r="M30" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.8329</t>
+          <t xml:space="preserve">0.8498</t>
         </is>
       </c>
       <c r="N30" t="inlineStr">
@@ -2426,7 +2414,7 @@
       </c>
       <c r="M31" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.6294</t>
+          <t xml:space="preserve">0.6554</t>
         </is>
       </c>
       <c r="N31" t="inlineStr">
@@ -2498,7 +2486,7 @@
       </c>
       <c r="M32" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.6221</t>
+          <t xml:space="preserve">0.649</t>
         </is>
       </c>
       <c r="N32" t="inlineStr">
@@ -2570,7 +2558,7 @@
       </c>
       <c r="M33" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.6356</t>
+          <t xml:space="preserve">0.793</t>
         </is>
       </c>
       <c r="N33" t="inlineStr">
@@ -2642,7 +2630,7 @@
       </c>
       <c r="M34" t="inlineStr">
         <is>
-          <t xml:space="preserve">4.4957</t>
+          <t xml:space="preserve">4.6176</t>
         </is>
       </c>
       <c r="N34" t="inlineStr">
@@ -2714,7 +2702,7 @@
       </c>
       <c r="M35" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.6227</t>
+          <t xml:space="preserve">0.6288</t>
         </is>
       </c>
       <c r="N35" t="inlineStr">
@@ -2786,7 +2774,7 @@
       </c>
       <c r="M36" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.8122</t>
+          <t xml:space="preserve">0.8319</t>
         </is>
       </c>
       <c r="N36" t="inlineStr">
@@ -2858,7 +2846,7 @@
       </c>
       <c r="M37" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.7429</t>
+          <t xml:space="preserve">0.6355</t>
         </is>
       </c>
       <c r="N37" t="inlineStr">
@@ -2930,7 +2918,7 @@
       </c>
       <c r="M38" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.6482</t>
+          <t xml:space="preserve">0.6637</t>
         </is>
       </c>
       <c r="N38" t="inlineStr">
@@ -3002,7 +2990,7 @@
       </c>
       <c r="M39" t="inlineStr">
         <is>
-          <t xml:space="preserve">2.5283</t>
+          <t xml:space="preserve">2.7492</t>
         </is>
       </c>
       <c r="N39" t="inlineStr">
@@ -3074,7 +3062,7 @@
       </c>
       <c r="M40" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.7338</t>
+          <t xml:space="preserve">0.6438</t>
         </is>
       </c>
       <c r="N40" t="inlineStr">
@@ -3146,7 +3134,7 @@
       </c>
       <c r="M41" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.625</t>
+          <t xml:space="preserve">0.6344</t>
         </is>
       </c>
       <c r="N41" t="inlineStr">
@@ -3218,7 +3206,7 @@
       </c>
       <c r="M42" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.6217</t>
+          <t xml:space="preserve">0.6564</t>
         </is>
       </c>
       <c r="N42" t="inlineStr">
@@ -3290,7 +3278,7 @@
       </c>
       <c r="M43" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.625</t>
+          <t xml:space="preserve">0.791</t>
         </is>
       </c>
       <c r="N43" t="inlineStr">
@@ -3362,7 +3350,7 @@
       </c>
       <c r="M44" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.4507</t>
+          <t xml:space="preserve">0.4633</t>
         </is>
       </c>
       <c r="N44" t="inlineStr">
@@ -3434,7 +3422,7 @@
       </c>
       <c r="M45" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.4655</t>
+          <t xml:space="preserve">0.4837</t>
         </is>
       </c>
       <c r="N45" t="inlineStr">
@@ -3506,7 +3494,7 @@
       </c>
       <c r="M46" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.4565</t>
+          <t xml:space="preserve">0.4578</t>
         </is>
       </c>
       <c r="N46" t="inlineStr">
@@ -3578,7 +3566,7 @@
       </c>
       <c r="M47" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.7488</t>
+          <t xml:space="preserve">0.6413</t>
         </is>
       </c>
       <c r="N47" t="inlineStr">
@@ -3650,7 +3638,7 @@
       </c>
       <c r="M48" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.4805</t>
+          <t xml:space="preserve">0.4894</t>
         </is>
       </c>
       <c r="N48" t="inlineStr">
@@ -3722,7 +3710,7 @@
       </c>
       <c r="M49" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.4867</t>
+          <t xml:space="preserve">0.4673</t>
         </is>
       </c>
       <c r="N49" t="inlineStr">
@@ -3794,7 +3782,7 @@
       </c>
       <c r="M50" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.8885</t>
+          <t xml:space="preserve">1.0198</t>
         </is>
       </c>
       <c r="N50" t="inlineStr">
@@ -3866,7 +3854,7 @@
       </c>
       <c r="M51" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.472</t>
+          <t xml:space="preserve">0.4831</t>
         </is>
       </c>
       <c r="N51" t="inlineStr">
@@ -3938,7 +3926,7 @@
       </c>
       <c r="M52" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.4844</t>
+          <t xml:space="preserve">0.5007</t>
         </is>
       </c>
       <c r="N52" t="inlineStr">
@@ -4010,7 +3998,7 @@
       </c>
       <c r="M53" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.5741</t>
+          <t xml:space="preserve">0.4752</t>
         </is>
       </c>
       <c r="N53" t="inlineStr">
@@ -4082,7 +4070,7 @@
       </c>
       <c r="M54" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.442</t>
+          <t xml:space="preserve">0.4525</t>
         </is>
       </c>
       <c r="N54" t="inlineStr">
@@ -4154,7 +4142,7 @@
       </c>
       <c r="M55" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.4767</t>
+          <t xml:space="preserve">0.6734</t>
         </is>
       </c>
       <c r="N55" t="inlineStr">
@@ -4226,7 +4214,7 @@
       </c>
       <c r="M56" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.0031</t>
+          <t xml:space="preserve">0.0033</t>
         </is>
       </c>
       <c r="N56" t="inlineStr">
@@ -4298,7 +4286,7 @@
       </c>
       <c r="M57" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.0036</t>
+          <t xml:space="preserve">0.0037</t>
         </is>
       </c>
       <c r="N57" t="inlineStr">
@@ -4370,7 +4358,7 @@
       </c>
       <c r="M58" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.003</t>
+          <t xml:space="preserve">0.0031</t>
         </is>
       </c>
       <c r="N58" t="inlineStr">
@@ -4442,7 +4430,7 @@
       </c>
       <c r="M59" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.0023</t>
+          <t xml:space="preserve">0.0025</t>
         </is>
       </c>
       <c r="N59" t="inlineStr">
@@ -4514,7 +4502,7 @@
       </c>
       <c r="M60" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.6393</t>
+          <t xml:space="preserve">0.6598</t>
         </is>
       </c>
       <c r="N60" t="inlineStr">
@@ -4586,7 +4574,7 @@
       </c>
       <c r="M61" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.0007</t>
+          <t xml:space="preserve">0.0008</t>
         </is>
       </c>
       <c r="N61" t="inlineStr">
@@ -4658,7 +4646,7 @@
       </c>
       <c r="M62" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.6153</t>
+          <t xml:space="preserve">0.6273</t>
         </is>
       </c>
       <c r="N62" t="inlineStr">
@@ -4730,7 +4718,7 @@
       </c>
       <c r="M63" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.6715</t>
+          <t xml:space="preserve">0.683</t>
         </is>
       </c>
       <c r="N63" t="inlineStr">
@@ -4802,7 +4790,7 @@
       </c>
       <c r="M64" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.7655</t>
+          <t xml:space="preserve">0.6896</t>
         </is>
       </c>
       <c r="N64" t="inlineStr">
@@ -4874,7 +4862,7 @@
       </c>
       <c r="M65" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.6591</t>
+          <t xml:space="preserve">0.6699</t>
         </is>
       </c>
       <c r="N65" t="inlineStr">
@@ -4946,7 +4934,7 @@
       </c>
       <c r="M66" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.6784</t>
+          <t xml:space="preserve">0.8468</t>
         </is>
       </c>
       <c r="N66" t="inlineStr">
@@ -5018,7 +5006,7 @@
       </c>
       <c r="M67" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.6691</t>
+          <t xml:space="preserve">0.6739</t>
         </is>
       </c>
       <c r="N67" t="inlineStr">
@@ -5090,7 +5078,7 @@
       </c>
       <c r="M68" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.6755</t>
+          <t xml:space="preserve">0.71</t>
         </is>
       </c>
       <c r="N68" t="inlineStr">
@@ -5162,7 +5150,7 @@
       </c>
       <c r="M69" t="inlineStr">
         <is>
-          <t xml:space="preserve">1.3342</t>
+          <t xml:space="preserve">1.4013</t>
         </is>
       </c>
       <c r="N69" t="inlineStr">
@@ -5234,7 +5222,7 @@
       </c>
       <c r="M70" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.8204</t>
+          <t xml:space="preserve">0.6969</t>
         </is>
       </c>
       <c r="N70" t="inlineStr">
@@ -5306,7 +5294,7 @@
       </c>
       <c r="M71" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.8161</t>
+          <t xml:space="preserve">0.9968</t>
         </is>
       </c>
       <c r="N71" t="inlineStr">
@@ -5378,7 +5366,7 @@
       </c>
       <c r="M72" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.7021</t>
+          <t xml:space="preserve">0.6901</t>
         </is>
       </c>
       <c r="N72" t="inlineStr">
@@ -5450,7 +5438,7 @@
       </c>
       <c r="M73" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.6136</t>
+          <t xml:space="preserve">0.6161</t>
         </is>
       </c>
       <c r="N73" t="inlineStr">
@@ -5522,7 +5510,7 @@
       </c>
       <c r="M74" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.4637</t>
+          <t xml:space="preserve">0.4755</t>
         </is>
       </c>
       <c r="N74" t="inlineStr">
@@ -5594,7 +5582,7 @@
       </c>
       <c r="M75" t="inlineStr">
         <is>
-          <t xml:space="preserve">3.3446</t>
+          <t xml:space="preserve">3.3493</t>
         </is>
       </c>
       <c r="N75" t="inlineStr">
@@ -5666,7 +5654,7 @@
       </c>
       <c r="M76" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.4486</t>
+          <t xml:space="preserve">0.4657</t>
         </is>
       </c>
       <c r="N76" t="inlineStr">
@@ -5738,7 +5726,7 @@
       </c>
       <c r="M77" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.6557</t>
+          <t xml:space="preserve">0.6584</t>
         </is>
       </c>
       <c r="N77" t="inlineStr">
@@ -5810,7 +5798,7 @@
       </c>
       <c r="M78" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.5009</t>
+          <t xml:space="preserve">0.4764</t>
         </is>
       </c>
       <c r="N78" t="inlineStr">
@@ -5882,7 +5870,7 @@
       </c>
       <c r="M79" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.6353</t>
+          <t xml:space="preserve">0.7739</t>
         </is>
       </c>
       <c r="N79" t="inlineStr">
@@ -5954,7 +5942,7 @@
       </c>
       <c r="M80" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.4694</t>
+          <t xml:space="preserve">0.4757</t>
         </is>
       </c>
       <c r="N80" t="inlineStr">
@@ -6026,7 +6014,7 @@
       </c>
       <c r="M81" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.4757</t>
+          <t xml:space="preserve">0.4908</t>
         </is>
       </c>
       <c r="N81" t="inlineStr">
@@ -6098,7 +6086,7 @@
       </c>
       <c r="M82" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.4582</t>
+          <t xml:space="preserve">0.4725</t>
         </is>
       </c>
       <c r="N82" t="inlineStr">
@@ -6170,7 +6158,7 @@
       </c>
       <c r="M83" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.6202</t>
+          <t xml:space="preserve">0.6351</t>
         </is>
       </c>
       <c r="N83" t="inlineStr">
@@ -6242,7 +6230,7 @@
       </c>
       <c r="M84" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.4916</t>
+          <t xml:space="preserve">0.5042</t>
         </is>
       </c>
       <c r="N84" t="inlineStr">
@@ -6314,7 +6302,7 @@
       </c>
       <c r="M85" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.6413</t>
+          <t xml:space="preserve">0.6621</t>
         </is>
       </c>
       <c r="N85" t="inlineStr">
@@ -6386,7 +6374,7 @@
       </c>
       <c r="M86" t="inlineStr">
         <is>
-          <t xml:space="preserve">1.2657</t>
+          <t xml:space="preserve">1.2968</t>
         </is>
       </c>
       <c r="N86" t="inlineStr">
@@ -6458,7 +6446,7 @@
       </c>
       <c r="M87" t="inlineStr">
         <is>
-          <t xml:space="preserve">4.7703</t>
+          <t xml:space="preserve">5.1123</t>
         </is>
       </c>
       <c r="N87" t="inlineStr">
@@ -6530,7 +6518,7 @@
       </c>
       <c r="M88" t="inlineStr">
         <is>
-          <t xml:space="preserve">1.0721</t>
+          <t xml:space="preserve">0.9074</t>
         </is>
       </c>
       <c r="N88" t="inlineStr">
@@ -6602,7 +6590,7 @@
       </c>
       <c r="M89" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.4407</t>
+          <t xml:space="preserve">0.4568</t>
         </is>
       </c>
       <c r="N89" t="inlineStr">
@@ -6674,7 +6662,7 @@
       </c>
       <c r="M90" t="inlineStr">
         <is>
-          <t xml:space="preserve">1.8239</t>
+          <t xml:space="preserve">2.0766</t>
         </is>
       </c>
       <c r="N90" t="inlineStr">
@@ -6746,7 +6734,7 @@
       </c>
       <c r="M91" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.4559</t>
+          <t xml:space="preserve">0.4676</t>
         </is>
       </c>
       <c r="N91" t="inlineStr">
@@ -6818,7 +6806,7 @@
       </c>
       <c r="M92" t="inlineStr">
         <is>
-          <t xml:space="preserve">3.3151</t>
+          <t xml:space="preserve">3.4395</t>
         </is>
       </c>
       <c r="N92" t="inlineStr">
@@ -6890,7 +6878,7 @@
       </c>
       <c r="M93" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.4503</t>
+          <t xml:space="preserve">0.4639</t>
         </is>
       </c>
       <c r="N93" t="inlineStr">
@@ -6962,7 +6950,7 @@
       </c>
       <c r="M94" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.8454</t>
+          <t xml:space="preserve">0.6423</t>
         </is>
       </c>
       <c r="N94" t="inlineStr">
@@ -7034,7 +7022,7 @@
       </c>
       <c r="M95" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.4694</t>
+          <t xml:space="preserve">0.4992</t>
         </is>
       </c>
       <c r="N95" t="inlineStr">
@@ -7106,7 +7094,7 @@
       </c>
       <c r="M96" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.4606</t>
+          <t xml:space="preserve">0.4731</t>
         </is>
       </c>
       <c r="N96" t="inlineStr">
@@ -7178,7 +7166,7 @@
       </c>
       <c r="M97" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.4978</t>
+          <t xml:space="preserve">0.4745</t>
         </is>
       </c>
       <c r="N97" t="inlineStr">
@@ -7250,7 +7238,7 @@
       </c>
       <c r="M98" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.8838</t>
+          <t xml:space="preserve">1.1069</t>
         </is>
       </c>
       <c r="N98" t="inlineStr">
@@ -7322,7 +7310,7 @@
       </c>
       <c r="M99" t="inlineStr">
         <is>
-          <t xml:space="preserve">1.4763</t>
+          <t xml:space="preserve">1.3552</t>
         </is>
       </c>
       <c r="N99" t="inlineStr">
@@ -7394,7 +7382,7 @@
       </c>
       <c r="M100" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.6494</t>
+          <t xml:space="preserve">0.6788</t>
         </is>
       </c>
       <c r="N100" t="inlineStr">
@@ -7466,7 +7454,7 @@
       </c>
       <c r="M101" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.4956</t>
+          <t xml:space="preserve">0.5672</t>
         </is>
       </c>
       <c r="N101" t="inlineStr">
@@ -7538,7 +7526,7 @@
       </c>
       <c r="M102" t="inlineStr">
         <is>
-          <t xml:space="preserve">1.3606</t>
+          <t xml:space="preserve">1.7043</t>
         </is>
       </c>
       <c r="N102" t="inlineStr">
@@ -7610,7 +7598,7 @@
       </c>
       <c r="M103" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.6125</t>
+          <t xml:space="preserve">0.5093</t>
         </is>
       </c>
       <c r="N103" t="inlineStr">
@@ -7682,7 +7670,7 @@
       </c>
       <c r="M104" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.4758</t>
+          <t xml:space="preserve">0.5648</t>
         </is>
       </c>
       <c r="N104" t="inlineStr">
@@ -7754,7 +7742,7 @@
       </c>
       <c r="M105" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.4557</t>
+          <t xml:space="preserve">0.4769</t>
         </is>
       </c>
       <c r="N105" t="inlineStr">
@@ -7826,7 +7814,7 @@
       </c>
       <c r="M106" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.6226</t>
+          <t xml:space="preserve">0.6397</t>
         </is>
       </c>
       <c r="N106" t="inlineStr">
@@ -7898,7 +7886,7 @@
       </c>
       <c r="M107" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.6265</t>
+          <t xml:space="preserve">0.888</t>
         </is>
       </c>
       <c r="N107" t="inlineStr">
@@ -7970,7 +7958,7 @@
       </c>
       <c r="M108" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.8178</t>
+          <t xml:space="preserve">0.8331</t>
         </is>
       </c>
       <c r="N108" t="inlineStr">
@@ -8042,7 +8030,7 @@
       </c>
       <c r="M109" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.6505</t>
+          <t xml:space="preserve">0.6667</t>
         </is>
       </c>
       <c r="N109" t="inlineStr">
@@ -8114,7 +8102,7 @@
       </c>
       <c r="M110" t="inlineStr">
         <is>
-          <t xml:space="preserve">2.7326</t>
+          <t xml:space="preserve">2.8702</t>
         </is>
       </c>
       <c r="N110" t="inlineStr">
@@ -8186,7 +8174,7 @@
       </c>
       <c r="M111" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.6451</t>
+          <t xml:space="preserve">0.6521</t>
         </is>
       </c>
       <c r="N111" t="inlineStr">
@@ -8258,7 +8246,7 @@
       </c>
       <c r="M112" t="inlineStr">
         <is>
-          <t xml:space="preserve">1.2808</t>
+          <t xml:space="preserve">1.3312</t>
         </is>
       </c>
       <c r="N112" t="inlineStr">
@@ -8330,7 +8318,7 @@
       </c>
       <c r="M113" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.8176</t>
+          <t xml:space="preserve">0.6606</t>
         </is>
       </c>
       <c r="N113" t="inlineStr">
@@ -8402,7 +8390,7 @@
       </c>
       <c r="M114" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.6687</t>
+          <t xml:space="preserve">0.6921</t>
         </is>
       </c>
       <c r="N114" t="inlineStr">
@@ -8474,7 +8462,7 @@
       </c>
       <c r="M115" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.6433</t>
+          <t xml:space="preserve">0.6662</t>
         </is>
       </c>
       <c r="N115" t="inlineStr">
@@ -8546,7 +8534,7 @@
       </c>
       <c r="M116" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.7468</t>
+          <t xml:space="preserve">0.9944</t>
         </is>
       </c>
       <c r="N116" t="inlineStr">
@@ -8618,7 +8606,7 @@
       </c>
       <c r="M117" t="inlineStr">
         <is>
-          <t xml:space="preserve">1.9335</t>
+          <t xml:space="preserve">1.9543</t>
         </is>
       </c>
       <c r="N117" t="inlineStr">
@@ -8690,7 +8678,7 @@
       </c>
       <c r="M118" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.6301</t>
+          <t xml:space="preserve">0.6663</t>
         </is>
       </c>
       <c r="N118" t="inlineStr">
@@ -8762,7 +8750,7 @@
       </c>
       <c r="M119" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.8328</t>
+          <t xml:space="preserve">0.6424</t>
         </is>
       </c>
       <c r="N119" t="inlineStr">
@@ -8834,7 +8822,7 @@
       </c>
       <c r="M120" t="inlineStr">
         <is>
-          <t xml:space="preserve">3.1484</t>
+          <t xml:space="preserve">3.5289</t>
         </is>
       </c>
       <c r="N120" t="inlineStr">
@@ -8906,7 +8894,7 @@
       </c>
       <c r="M121" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.796</t>
+          <t xml:space="preserve">0.8156</t>
         </is>
       </c>
       <c r="N121" t="inlineStr">
@@ -8978,7 +8966,7 @@
       </c>
       <c r="M122" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.0004</t>
+          <t xml:space="preserve">0.0005</t>
         </is>
       </c>
       <c r="N122" t="inlineStr">
@@ -9050,7 +9038,7 @@
       </c>
       <c r="M123" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.6223</t>
+          <t xml:space="preserve">0.6433</t>
         </is>
       </c>
       <c r="N123" t="inlineStr">
@@ -9122,7 +9110,7 @@
       </c>
       <c r="M124" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.0006</t>
+          <t xml:space="preserve">0.0009</t>
         </is>
       </c>
       <c r="N124" t="inlineStr">
@@ -9194,7 +9182,7 @@
       </c>
       <c r="M125" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.6474</t>
+          <t xml:space="preserve">0.6748</t>
         </is>
       </c>
       <c r="N125" t="inlineStr">
@@ -9266,7 +9254,7 @@
       </c>
       <c r="M126" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.6246</t>
+          <t xml:space="preserve">0.6664</t>
         </is>
       </c>
       <c r="N126" t="inlineStr">
@@ -9338,7 +9326,7 @@
       </c>
       <c r="M127" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.6273</t>
+          <t xml:space="preserve">0.6624</t>
         </is>
       </c>
       <c r="N127" t="inlineStr">
@@ -9410,7 +9398,7 @@
       </c>
       <c r="M128" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.0004</t>
+          <t xml:space="preserve">0.0006</t>
         </is>
       </c>
       <c r="N128" t="inlineStr">
@@ -9482,7 +9470,7 @@
       </c>
       <c r="M129" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.6746</t>
+          <t xml:space="preserve">0.7202</t>
         </is>
       </c>
       <c r="N129" t="inlineStr">
@@ -9554,7 +9542,7 @@
       </c>
       <c r="M130" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.001</t>
+          <t xml:space="preserve">0.0007</t>
         </is>
       </c>
       <c r="N130" t="inlineStr">
@@ -9563,8 +9551,944 @@
         </is>
       </c>
     </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t xml:space="preserve">130</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t xml:space="preserve">UT-130</t>
+        </is>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t xml:space="preserve">REQ-QUALITY-LIFECYCLE</t>
+        </is>
+      </c>
+      <c r="D131" t="inlineStr">
+        <is>
+          <t xml:space="preserve">quality_lifecycle</t>
+        </is>
+      </c>
+      <c r="E131" t="inlineStr">
+        <is>
+          <t xml:space="preserve">API·단위/흐름</t>
+        </is>
+      </c>
+      <c r="F131" t="inlineStr">
+        <is>
+          <t xml:space="preserve">전체 학습·평가 샘플 검수</t>
+        </is>
+      </c>
+      <c r="G131" t="inlineStr">
+        <is>
+          <t xml:space="preserve">실제 GPU·유료 API 미사용; 파일과 모델 응답은 테스트용</t>
+        </is>
+      </c>
+      <c r="H131" t="inlineStr">
+        <is>
+          <t xml:space="preserve">임시 DB·합성 샘플·모사 모델로 성공·실패 및 저장 상태 확인</t>
+        </is>
+      </c>
+      <c r="I131" t="inlineStr">
+        <is>
+          <t xml:space="preserve">전체 검수·고정 평가·후보 검증·접근 제어 기준 충족</t>
+        </is>
+      </c>
+      <c r="J131" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tests/test_quality_lifecycle.py::test_full_review_covers_train_and_eval</t>
+        </is>
+      </c>
+      <c r="K131" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PASS</t>
+        </is>
+      </c>
+      <c r="L131" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1</t>
+        </is>
+      </c>
+      <c r="M131" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0.6469</t>
+        </is>
+      </c>
+      <c r="N131" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t xml:space="preserve">131</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t xml:space="preserve">UT-131</t>
+        </is>
+      </c>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t xml:space="preserve">REQ-QUALITY-LIFECYCLE</t>
+        </is>
+      </c>
+      <c r="D132" t="inlineStr">
+        <is>
+          <t xml:space="preserve">quality_lifecycle</t>
+        </is>
+      </c>
+      <c r="E132" t="inlineStr">
+        <is>
+          <t xml:space="preserve">API·단위/흐름</t>
+        </is>
+      </c>
+      <c r="F132" t="inlineStr">
+        <is>
+          <t xml:space="preserve">거부·위험·비정상응답 차단</t>
+        </is>
+      </c>
+      <c r="G132" t="inlineStr">
+        <is>
+          <t xml:space="preserve">실제 GPU·유료 API 미사용; 파일과 모델 응답은 테스트용</t>
+        </is>
+      </c>
+      <c r="H132" t="inlineStr">
+        <is>
+          <t xml:space="preserve">임시 DB·합성 샘플·모사 모델로 성공·실패 및 저장 상태 확인</t>
+        </is>
+      </c>
+      <c r="I132" t="inlineStr">
+        <is>
+          <t xml:space="preserve">전체 검수·고정 평가·후보 검증·접근 제어 기준 충족</t>
+        </is>
+      </c>
+      <c r="J132" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tests/test_quality_lifecycle.py::test_full_review_rejects_or_fails_closed</t>
+        </is>
+      </c>
+      <c r="K132" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PASS</t>
+        </is>
+      </c>
+      <c r="L132" t="inlineStr">
+        <is>
+          <t xml:space="preserve">5</t>
+        </is>
+      </c>
+      <c r="M132" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0.0043</t>
+        </is>
+      </c>
+      <c r="N132" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t xml:space="preserve">132</t>
+        </is>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t xml:space="preserve">UT-132</t>
+        </is>
+      </c>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t xml:space="preserve">REQ-QUALITY-LIFECYCLE</t>
+        </is>
+      </c>
+      <c r="D133" t="inlineStr">
+        <is>
+          <t xml:space="preserve">quality_lifecycle</t>
+        </is>
+      </c>
+      <c r="E133" t="inlineStr">
+        <is>
+          <t xml:space="preserve">API·단위/흐름</t>
+        </is>
+      </c>
+      <c r="F133" t="inlineStr">
+        <is>
+          <t xml:space="preserve">검수 중 오류 부분 통과 방지</t>
+        </is>
+      </c>
+      <c r="G133" t="inlineStr">
+        <is>
+          <t xml:space="preserve">실제 GPU·유료 API 미사용; 파일과 모델 응답은 테스트용</t>
+        </is>
+      </c>
+      <c r="H133" t="inlineStr">
+        <is>
+          <t xml:space="preserve">임시 DB·합성 샘플·모사 모델로 성공·실패 및 저장 상태 확인</t>
+        </is>
+      </c>
+      <c r="I133" t="inlineStr">
+        <is>
+          <t xml:space="preserve">전체 검수·고정 평가·후보 검증·접근 제어 기준 충족</t>
+        </is>
+      </c>
+      <c r="J133" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tests/test_quality_lifecycle.py::test_review_error_does_not_store_partial_pass</t>
+        </is>
+      </c>
+      <c r="K133" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PASS</t>
+        </is>
+      </c>
+      <c r="L133" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1</t>
+        </is>
+      </c>
+      <c r="M133" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1.0526</t>
+        </is>
+      </c>
+      <c r="N133" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t xml:space="preserve">133</t>
+        </is>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t xml:space="preserve">UT-133</t>
+        </is>
+      </c>
+      <c r="C134" t="inlineStr">
+        <is>
+          <t xml:space="preserve">REQ-QUALITY-LIFECYCLE</t>
+        </is>
+      </c>
+      <c r="D134" t="inlineStr">
+        <is>
+          <t xml:space="preserve">quality_lifecycle</t>
+        </is>
+      </c>
+      <c r="E134" t="inlineStr">
+        <is>
+          <t xml:space="preserve">API·단위/흐름</t>
+        </is>
+      </c>
+      <c r="F134" t="inlineStr">
+        <is>
+          <t xml:space="preserve">기존 3개 검수 재승인 차단</t>
+        </is>
+      </c>
+      <c r="G134" t="inlineStr">
+        <is>
+          <t xml:space="preserve">실제 GPU·유료 API 미사용; 파일과 모델 응답은 테스트용</t>
+        </is>
+      </c>
+      <c r="H134" t="inlineStr">
+        <is>
+          <t xml:space="preserve">임시 DB·합성 샘플·모사 모델로 성공·실패 및 저장 상태 확인</t>
+        </is>
+      </c>
+      <c r="I134" t="inlineStr">
+        <is>
+          <t xml:space="preserve">전체 검수·고정 평가·후보 검증·접근 제어 기준 충족</t>
+        </is>
+      </c>
+      <c r="J134" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tests/test_quality_lifecycle.py::test_old_preview_cannot_approve</t>
+        </is>
+      </c>
+      <c r="K134" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PASS</t>
+        </is>
+      </c>
+      <c r="L134" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1</t>
+        </is>
+      </c>
+      <c r="M134" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0.7443</t>
+        </is>
+      </c>
+      <c r="N134" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t xml:space="preserve">134</t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t xml:space="preserve">UT-134</t>
+        </is>
+      </c>
+      <c r="C135" t="inlineStr">
+        <is>
+          <t xml:space="preserve">REQ-QUALITY-LIFECYCLE</t>
+        </is>
+      </c>
+      <c r="D135" t="inlineStr">
+        <is>
+          <t xml:space="preserve">quality_lifecycle</t>
+        </is>
+      </c>
+      <c r="E135" t="inlineStr">
+        <is>
+          <t xml:space="preserve">API·단위/흐름</t>
+        </is>
+      </c>
+      <c r="F135" t="inlineStr">
+        <is>
+          <t xml:space="preserve">고정 평가·승인 해시 연결</t>
+        </is>
+      </c>
+      <c r="G135" t="inlineStr">
+        <is>
+          <t xml:space="preserve">실제 GPU·유료 API 미사용; 파일과 모델 응답은 테스트용</t>
+        </is>
+      </c>
+      <c r="H135" t="inlineStr">
+        <is>
+          <t xml:space="preserve">임시 DB·합성 샘플·모사 모델로 성공·실패 및 저장 상태 확인</t>
+        </is>
+      </c>
+      <c r="I135" t="inlineStr">
+        <is>
+          <t xml:space="preserve">전체 검수·고정 평가·후보 검증·접근 제어 기준 충족</t>
+        </is>
+      </c>
+      <c r="J135" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tests/test_quality_lifecycle.py::test_benchmark_registration_and_immutable_plan</t>
+        </is>
+      </c>
+      <c r="K135" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PASS</t>
+        </is>
+      </c>
+      <c r="L135" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1</t>
+        </is>
+      </c>
+      <c r="M135" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0.6876</t>
+        </is>
+      </c>
+      <c r="N135" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t xml:space="preserve">135</t>
+        </is>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t xml:space="preserve">UT-135</t>
+        </is>
+      </c>
+      <c r="C136" t="inlineStr">
+        <is>
+          <t xml:space="preserve">REQ-QUALITY-LIFECYCLE</t>
+        </is>
+      </c>
+      <c r="D136" t="inlineStr">
+        <is>
+          <t xml:space="preserve">quality_lifecycle</t>
+        </is>
+      </c>
+      <c r="E136" t="inlineStr">
+        <is>
+          <t xml:space="preserve">API·단위/흐름</t>
+        </is>
+      </c>
+      <c r="F136" t="inlineStr">
+        <is>
+          <t xml:space="preserve">평가 입력 제한·중복</t>
+        </is>
+      </c>
+      <c r="G136" t="inlineStr">
+        <is>
+          <t xml:space="preserve">실제 GPU·유료 API 미사용; 파일과 모델 응답은 테스트용</t>
+        </is>
+      </c>
+      <c r="H136" t="inlineStr">
+        <is>
+          <t xml:space="preserve">임시 DB·합성 샘플·모사 모델로 성공·실패 및 저장 상태 확인</t>
+        </is>
+      </c>
+      <c r="I136" t="inlineStr">
+        <is>
+          <t xml:space="preserve">전체 검수·고정 평가·후보 검증·접근 제어 기준 충족</t>
+        </is>
+      </c>
+      <c r="J136" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tests/test_quality_lifecycle.py::test_benchmark_limits_and_duplicates</t>
+        </is>
+      </c>
+      <c r="K136" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PASS</t>
+        </is>
+      </c>
+      <c r="L136" t="inlineStr">
+        <is>
+          <t xml:space="preserve">3</t>
+        </is>
+      </c>
+      <c r="M136" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1.8878</t>
+        </is>
+      </c>
+      <c r="N136" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t xml:space="preserve">136</t>
+        </is>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t xml:space="preserve">UT-136</t>
+        </is>
+      </c>
+      <c r="C137" t="inlineStr">
+        <is>
+          <t xml:space="preserve">REQ-QUALITY-LIFECYCLE</t>
+        </is>
+      </c>
+      <c r="D137" t="inlineStr">
+        <is>
+          <t xml:space="preserve">quality_lifecycle</t>
+        </is>
+      </c>
+      <c r="E137" t="inlineStr">
+        <is>
+          <t xml:space="preserve">API·단위/흐름</t>
+        </is>
+      </c>
+      <c r="F137" t="inlineStr">
+        <is>
+          <t xml:space="preserve">학습 문항 유출·미등록 평가 차단</t>
+        </is>
+      </c>
+      <c r="G137" t="inlineStr">
+        <is>
+          <t xml:space="preserve">실제 GPU·유료 API 미사용; 파일과 모델 응답은 테스트용</t>
+        </is>
+      </c>
+      <c r="H137" t="inlineStr">
+        <is>
+          <t xml:space="preserve">임시 DB·합성 샘플·모사 모델로 성공·실패 및 저장 상태 확인</t>
+        </is>
+      </c>
+      <c r="I137" t="inlineStr">
+        <is>
+          <t xml:space="preserve">전체 검수·고정 평가·후보 검증·접근 제어 기준 충족</t>
+        </is>
+      </c>
+      <c r="J137" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tests/test_quality_lifecycle.py::test_benchmark_leakage_and_unknown_suite</t>
+        </is>
+      </c>
+      <c r="K137" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PASS</t>
+        </is>
+      </c>
+      <c r="L137" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1</t>
+        </is>
+      </c>
+      <c r="M137" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0.6858</t>
+        </is>
+      </c>
+      <c r="N137" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t xml:space="preserve">137</t>
+        </is>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t xml:space="preserve">UT-137</t>
+        </is>
+      </c>
+      <c r="C138" t="inlineStr">
+        <is>
+          <t xml:space="preserve">REQ-QUALITY-LIFECYCLE</t>
+        </is>
+      </c>
+      <c r="D138" t="inlineStr">
+        <is>
+          <t xml:space="preserve">quality_lifecycle</t>
+        </is>
+      </c>
+      <c r="E138" t="inlineStr">
+        <is>
+          <t xml:space="preserve">API·단위/흐름</t>
+        </is>
+      </c>
+      <c r="F138" t="inlineStr">
+        <is>
+          <t xml:space="preserve">정답 정규화·응답 검증</t>
+        </is>
+      </c>
+      <c r="G138" t="inlineStr">
+        <is>
+          <t xml:space="preserve">실제 GPU·유료 API 미사용; 파일과 모델 응답은 테스트용</t>
+        </is>
+      </c>
+      <c r="H138" t="inlineStr">
+        <is>
+          <t xml:space="preserve">임시 DB·합성 샘플·모사 모델로 성공·실패 및 저장 상태 확인</t>
+        </is>
+      </c>
+      <c r="I138" t="inlineStr">
+        <is>
+          <t xml:space="preserve">전체 검수·고정 평가·후보 검증·접근 제어 기준 충족</t>
+        </is>
+      </c>
+      <c r="J138" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tests/test_quality_lifecycle.py::test_benchmark_exact_match_and_response_validation</t>
+        </is>
+      </c>
+      <c r="K138" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PASS</t>
+        </is>
+      </c>
+      <c r="L138" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1</t>
+        </is>
+      </c>
+      <c r="M138" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0.0109</t>
+        </is>
+      </c>
+      <c r="N138" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t xml:space="preserve">138</t>
+        </is>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t xml:space="preserve">UT-138</t>
+        </is>
+      </c>
+      <c r="C139" t="inlineStr">
+        <is>
+          <t xml:space="preserve">REQ-QUALITY-LIFECYCLE</t>
+        </is>
+      </c>
+      <c r="D139" t="inlineStr">
+        <is>
+          <t xml:space="preserve">quality_lifecycle</t>
+        </is>
+      </c>
+      <c r="E139" t="inlineStr">
+        <is>
+          <t xml:space="preserve">API·단위/흐름</t>
+        </is>
+      </c>
+      <c r="F139" t="inlineStr">
+        <is>
+          <t xml:space="preserve">통합 상태·가짜 진행률 방지</t>
+        </is>
+      </c>
+      <c r="G139" t="inlineStr">
+        <is>
+          <t xml:space="preserve">실제 GPU·유료 API 미사용; 파일과 모델 응답은 테스트용</t>
+        </is>
+      </c>
+      <c r="H139" t="inlineStr">
+        <is>
+          <t xml:space="preserve">임시 DB·합성 샘플·모사 모델로 성공·실패 및 저장 상태 확인</t>
+        </is>
+      </c>
+      <c r="I139" t="inlineStr">
+        <is>
+          <t xml:space="preserve">전체 검수·고정 평가·후보 검증·접근 제어 기준 충족</t>
+        </is>
+      </c>
+      <c r="J139" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tests/test_quality_lifecycle.py::test_dashboard_no_worker_or_percent_claim</t>
+        </is>
+      </c>
+      <c r="K139" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PASS</t>
+        </is>
+      </c>
+      <c r="L139" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1</t>
+        </is>
+      </c>
+      <c r="M139" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0.7286</t>
+        </is>
+      </c>
+      <c r="N139" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t xml:space="preserve">139</t>
+        </is>
+      </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t xml:space="preserve">UT-139</t>
+        </is>
+      </c>
+      <c r="C140" t="inlineStr">
+        <is>
+          <t xml:space="preserve">REQ-QUALITY-LIFECYCLE</t>
+        </is>
+      </c>
+      <c r="D140" t="inlineStr">
+        <is>
+          <t xml:space="preserve">quality_lifecycle</t>
+        </is>
+      </c>
+      <c r="E140" t="inlineStr">
+        <is>
+          <t xml:space="preserve">API·단위/흐름</t>
+        </is>
+      </c>
+      <c r="F140" t="inlineStr">
+        <is>
+          <t xml:space="preserve">후보 선택·롤백·동시 변경</t>
+        </is>
+      </c>
+      <c r="G140" t="inlineStr">
+        <is>
+          <t xml:space="preserve">실제 GPU·유료 API 미사용; 파일과 모델 응답은 테스트용</t>
+        </is>
+      </c>
+      <c r="H140" t="inlineStr">
+        <is>
+          <t xml:space="preserve">임시 DB·합성 샘플·모사 모델로 성공·실패 및 저장 상태 확인</t>
+        </is>
+      </c>
+      <c r="I140" t="inlineStr">
+        <is>
+          <t xml:space="preserve">전체 검수·고정 평가·후보 검증·접근 제어 기준 충족</t>
+        </is>
+      </c>
+      <c r="J140" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tests/test_quality_lifecycle.py::test_candidate_selection_rollback_and_cas</t>
+        </is>
+      </c>
+      <c r="K140" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PASS</t>
+        </is>
+      </c>
+      <c r="L140" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1</t>
+        </is>
+      </c>
+      <c r="M140" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0.7776</t>
+        </is>
+      </c>
+      <c r="N140" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t xml:space="preserve">140</t>
+        </is>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t xml:space="preserve">UT-140</t>
+        </is>
+      </c>
+      <c r="C141" t="inlineStr">
+        <is>
+          <t xml:space="preserve">REQ-QUALITY-LIFECYCLE</t>
+        </is>
+      </c>
+      <c r="D141" t="inlineStr">
+        <is>
+          <t xml:space="preserve">quality_lifecycle</t>
+        </is>
+      </c>
+      <c r="E141" t="inlineStr">
+        <is>
+          <t xml:space="preserve">API·단위/흐름</t>
+        </is>
+      </c>
+      <c r="F141" t="inlineStr">
+        <is>
+          <t xml:space="preserve">변조·퇴행·평가누락·가짜학습 차단</t>
+        </is>
+      </c>
+      <c r="G141" t="inlineStr">
+        <is>
+          <t xml:space="preserve">실제 GPU·유료 API 미사용; 파일과 모델 응답은 테스트용</t>
+        </is>
+      </c>
+      <c r="H141" t="inlineStr">
+        <is>
+          <t xml:space="preserve">임시 DB·합성 샘플·모사 모델로 성공·실패 및 저장 상태 확인</t>
+        </is>
+      </c>
+      <c r="I141" t="inlineStr">
+        <is>
+          <t xml:space="preserve">전체 검수·고정 평가·후보 검증·접근 제어 기준 충족</t>
+        </is>
+      </c>
+      <c r="J141" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tests/test_quality_lifecycle.py::test_candidate_validation_blocks_bad_versions</t>
+        </is>
+      </c>
+      <c r="K141" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PASS</t>
+        </is>
+      </c>
+      <c r="L141" t="inlineStr">
+        <is>
+          <t xml:space="preserve">4</t>
+        </is>
+      </c>
+      <c r="M141" t="inlineStr">
+        <is>
+          <t xml:space="preserve">3.2751</t>
+        </is>
+      </c>
+      <c r="N141" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t xml:space="preserve">141</t>
+        </is>
+      </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t xml:space="preserve">UT-141</t>
+        </is>
+      </c>
+      <c r="C142" t="inlineStr">
+        <is>
+          <t xml:space="preserve">REQ-QUALITY-LIFECYCLE</t>
+        </is>
+      </c>
+      <c r="D142" t="inlineStr">
+        <is>
+          <t xml:space="preserve">quality_lifecycle</t>
+        </is>
+      </c>
+      <c r="E142" t="inlineStr">
+        <is>
+          <t xml:space="preserve">API·단위/흐름</t>
+        </is>
+      </c>
+      <c r="F142" t="inlineStr">
+        <is>
+          <t xml:space="preserve">롤백 이전 파일 재검증</t>
+        </is>
+      </c>
+      <c r="G142" t="inlineStr">
+        <is>
+          <t xml:space="preserve">실제 GPU·유료 API 미사용; 파일과 모델 응답은 테스트용</t>
+        </is>
+      </c>
+      <c r="H142" t="inlineStr">
+        <is>
+          <t xml:space="preserve">임시 DB·합성 샘플·모사 모델로 성공·실패 및 저장 상태 확인</t>
+        </is>
+      </c>
+      <c r="I142" t="inlineStr">
+        <is>
+          <t xml:space="preserve">전체 검수·고정 평가·후보 검증·접근 제어 기준 충족</t>
+        </is>
+      </c>
+      <c r="J142" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tests/test_quality_lifecycle.py::test_rollback_revalidates_previous_files</t>
+        </is>
+      </c>
+      <c r="K142" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PASS</t>
+        </is>
+      </c>
+      <c r="L142" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1</t>
+        </is>
+      </c>
+      <c r="M142" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0.7837</t>
+        </is>
+      </c>
+      <c r="N142" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t xml:space="preserve">142</t>
+        </is>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t xml:space="preserve">UT-142</t>
+        </is>
+      </c>
+      <c r="C143" t="inlineStr">
+        <is>
+          <t xml:space="preserve">REQ-QUALITY-LIFECYCLE</t>
+        </is>
+      </c>
+      <c r="D143" t="inlineStr">
+        <is>
+          <t xml:space="preserve">quality_lifecycle</t>
+        </is>
+      </c>
+      <c r="E143" t="inlineStr">
+        <is>
+          <t xml:space="preserve">API·단위/흐름</t>
+        </is>
+      </c>
+      <c r="F143" t="inlineStr">
+        <is>
+          <t xml:space="preserve">소유자·CSRF 제한</t>
+        </is>
+      </c>
+      <c r="G143" t="inlineStr">
+        <is>
+          <t xml:space="preserve">실제 GPU·유료 API 미사용; 파일과 모델 응답은 테스트용</t>
+        </is>
+      </c>
+      <c r="H143" t="inlineStr">
+        <is>
+          <t xml:space="preserve">임시 DB·합성 샘플·모사 모델로 성공·실패 및 저장 상태 확인</t>
+        </is>
+      </c>
+      <c r="I143" t="inlineStr">
+        <is>
+          <t xml:space="preserve">전체 검수·고정 평가·후보 검증·접근 제어 기준 충족</t>
+        </is>
+      </c>
+      <c r="J143" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tests/test_quality_lifecycle.py::test_lifecycle_owner_and_csrf</t>
+        </is>
+      </c>
+      <c r="K143" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PASS</t>
+        </is>
+      </c>
+      <c r="L143" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1</t>
+        </is>
+      </c>
+      <c r="M143" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0.815</t>
+        </is>
+      </c>
+      <c r="N143" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:N130"/>
+  <autoFilter ref="A1:N143"/>
 </worksheet>
 </file>
 
@@ -9877,8 +10801,25 @@
         </is>
       </c>
     </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">전체검수·고정평가·배포후보·통합현황</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">행별 로컬검수/학습계획 평가 고정/파일 검증/후보 롤백/권한</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">자동 검증; 실제 GPU 생성·배포는 별도</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:C18"/>
+  <autoFilter ref="A1:C19"/>
 </worksheet>
 </file>
 
@@ -10105,8 +11046,30 @@
         </is>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ENV-QUALITY</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">전체 검수·GPU 전후 고정 질문 생성</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">실제 Ollama 및 기반 모델·GPU</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">미실행</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:D10"/>
+  <autoFilter ref="A1:D11"/>
 </worksheet>
 </file>
 
@@ -10163,7 +11126,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t xml:space="preserve">PASS / https://github.com/wjdwodhks35/Role-AI/actions/runs/38536591380</t>
+          <t xml:space="preserve">PASS / https://github.com/wjdwodhks35/Role-AI/actions/runs/38539414117</t>
         </is>
       </c>
     </row>
@@ -10190,66 +11153,39 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t xml:space="preserve">PASS / https://github.com/wjdwodhks35/Role-AI/actions/runs/38536591380</t>
+          <t xml:space="preserve">PASS / https://github.com/wjdwodhks35/Role-AI/actions/runs/38539414117</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t xml:space="preserve">QA-GPU-001</t>
+          <t xml:space="preserve">CI-QUALITY-001</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t xml:space="preserve">정적검사</t>
+          <t xml:space="preserve">코드 검사</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Fixture import shadowing F811 / https://github.com/wjdwodhks35/Role-AI/actions/runs/38536109299</t>
+          <t xml:space="preserve">unused import json / Actions 38539290960</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t xml:space="preserve">공유 pytest fixture 별칭 등록</t>
+          <t xml:space="preserve">불필요한 import 제거</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t xml:space="preserve">정적검사 및 전체테스트 PASS / https://github.com/wjdwodhks35/Role-AI/actions/runs/38536591380</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">CONFIG-001</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">수집 Worker 상태검사</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">구성 점검: CLI Worker가 웹HTTP healthcheck를 상속</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">수집 서비스 HTTP healthcheck 비활성화</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">최종 Compose 검증 대기; 실제GPUWorker 미실행</t>
+          <t xml:space="preserve">PASS / https://github.com/wjdwodhks35/Role-AI/actions/runs/38539414117</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E5"/>
+  <autoFilter ref="A1:E4"/>
 </worksheet>
 </file>
 
@@ -10259,7 +11195,7 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t xml:space="preserve">실행순서</t>
+          <t xml:space="preserve">순서</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
@@ -10286,7 +11222,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t xml:space="preserve">PASS</t>
+          <t xml:space="preserve">PASS (CI 요구사항 실행 결과; 단계별 내역은 CI artifact 참조)</t>
         </is>
       </c>
     </row>
@@ -10303,7 +11239,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t xml:space="preserve">PASS</t>
+          <t xml:space="preserve">PASS (CI 요구사항 실행 결과; 단계별 내역은 CI artifact 참조)</t>
         </is>
       </c>
     </row>
@@ -10320,7 +11256,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t xml:space="preserve">PASS</t>
+          <t xml:space="preserve">PASS (CI 요구사항 실행 결과; 단계별 내역은 CI artifact 참조)</t>
         </is>
       </c>
     </row>
@@ -10337,7 +11273,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t xml:space="preserve">PASS</t>
+          <t xml:space="preserve">PASS (CI 요구사항 실행 결과; 단계별 내역은 CI artifact 참조)</t>
         </is>
       </c>
     </row>
@@ -10354,7 +11290,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t xml:space="preserve">PASS</t>
+          <t xml:space="preserve">PASS (CI 요구사항 실행 결과; 단계별 내역은 CI artifact 참조)</t>
         </is>
       </c>
     </row>
@@ -10371,7 +11307,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t xml:space="preserve">PASS</t>
+          <t xml:space="preserve">PASS (CI 요구사항 실행 결과; 단계별 내역은 CI artifact 참조)</t>
         </is>
       </c>
     </row>
@@ -10388,7 +11324,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t xml:space="preserve">PASS</t>
+          <t xml:space="preserve">PASS (CI 요구사항 실행 결과; 단계별 내역은 CI artifact 참조)</t>
         </is>
       </c>
     </row>
@@ -10405,7 +11341,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t xml:space="preserve">PASS</t>
+          <t xml:space="preserve">PASS (CI 요구사항 실행 결과; 단계별 내역은 CI artifact 참조)</t>
         </is>
       </c>
     </row>
@@ -10422,7 +11358,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t xml:space="preserve">PASS</t>
+          <t xml:space="preserve">PASS (CI 요구사항 실행 결과; 단계별 내역은 CI artifact 참조)</t>
         </is>
       </c>
     </row>
@@ -10439,7 +11375,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t xml:space="preserve">PASS</t>
+          <t xml:space="preserve">PASS (CI 요구사항 실행 결과; 단계별 내역은 CI artifact 참조)</t>
         </is>
       </c>
     </row>
@@ -10456,7 +11392,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t xml:space="preserve">PASS</t>
+          <t xml:space="preserve">PASS (CI 요구사항 실행 결과; 단계별 내역은 CI artifact 참조)</t>
         </is>
       </c>
     </row>
@@ -10473,7 +11409,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t xml:space="preserve">PASS</t>
+          <t xml:space="preserve">PASS (CI 요구사항 실행 결과; 단계별 내역은 CI artifact 참조)</t>
         </is>
       </c>
     </row>
@@ -10490,7 +11426,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t xml:space="preserve">PASS</t>
+          <t xml:space="preserve">PASS (CI 요구사항 실행 결과; 단계별 내역은 CI artifact 참조)</t>
         </is>
       </c>
     </row>
@@ -10507,7 +11443,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t xml:space="preserve">PASS</t>
+          <t xml:space="preserve">PASS (CI 요구사항 실행 결과; 단계별 내역은 CI artifact 참조)</t>
         </is>
       </c>
     </row>
@@ -10524,7 +11460,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t xml:space="preserve">PASS</t>
+          <t xml:space="preserve">PASS (CI 요구사항 실행 결과; 단계별 내역은 CI artifact 참조)</t>
         </is>
       </c>
     </row>
@@ -10541,7 +11477,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t xml:space="preserve">PASS</t>
+          <t xml:space="preserve">PASS (CI 요구사항 실행 결과; 단계별 내역은 CI artifact 참조)</t>
         </is>
       </c>
     </row>
@@ -10558,7 +11494,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t xml:space="preserve">PASS</t>
+          <t xml:space="preserve">PASS (CI 요구사항 실행 결과; 단계별 내역은 CI artifact 참조)</t>
         </is>
       </c>
     </row>
@@ -10575,7 +11511,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t xml:space="preserve">PASS</t>
+          <t xml:space="preserve">PASS (CI 요구사항 실행 결과; 단계별 내역은 CI artifact 참조)</t>
         </is>
       </c>
     </row>
@@ -10592,7 +11528,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t xml:space="preserve">PASS</t>
+          <t xml:space="preserve">PASS (CI 요구사항 실행 결과; 단계별 내역은 CI artifact 참조)</t>
         </is>
       </c>
     </row>
@@ -10609,7 +11545,7 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t xml:space="preserve">PASS</t>
+          <t xml:space="preserve">PASS (CI 요구사항 실행 결과; 단계별 내역은 CI artifact 참조)</t>
         </is>
       </c>
     </row>
@@ -10626,7 +11562,7 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t xml:space="preserve">PASS</t>
+          <t xml:space="preserve">PASS (CI 요구사항 실행 결과; 단계별 내역은 CI artifact 참조)</t>
         </is>
       </c>
     </row>
@@ -10643,7 +11579,7 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t xml:space="preserve">PASS</t>
+          <t xml:space="preserve">PASS (CI 요구사항 실행 결과; 단계별 내역은 CI artifact 참조)</t>
         </is>
       </c>
     </row>
@@ -10660,7 +11596,7 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t xml:space="preserve">PASS</t>
+          <t xml:space="preserve">PASS (CI 요구사항 실행 결과; 단계별 내역은 CI artifact 참조)</t>
         </is>
       </c>
     </row>
@@ -10677,7 +11613,7 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t xml:space="preserve">PASS</t>
+          <t xml:space="preserve">PASS (CI 요구사항 실행 결과; 단계별 내역은 CI artifact 참조)</t>
         </is>
       </c>
     </row>
@@ -10694,7 +11630,7 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t xml:space="preserve">PASS</t>
+          <t xml:space="preserve">PASS (CI 요구사항 실행 결과; 단계별 내역은 CI artifact 참조)</t>
         </is>
       </c>
     </row>
@@ -10711,7 +11647,7 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t xml:space="preserve">PASS</t>
+          <t xml:space="preserve">PASS (CI 요구사항 실행 결과; 단계별 내역은 CI artifact 참조)</t>
         </is>
       </c>
     </row>
@@ -10728,7 +11664,7 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t xml:space="preserve">PASS</t>
+          <t xml:space="preserve">PASS (CI 요구사항 실행 결과; 단계별 내역은 CI artifact 참조)</t>
         </is>
       </c>
     </row>
@@ -10745,7 +11681,7 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t xml:space="preserve">PASS</t>
+          <t xml:space="preserve">PASS (CI 요구사항 실행 결과; 단계별 내역은 CI artifact 참조)</t>
         </is>
       </c>
     </row>
@@ -10762,7 +11698,7 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t xml:space="preserve">PASS</t>
+          <t xml:space="preserve">PASS (CI 요구사항 실행 결과; 단계별 내역은 CI artifact 참조)</t>
         </is>
       </c>
     </row>
@@ -10779,7 +11715,7 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t xml:space="preserve">PASS</t>
+          <t xml:space="preserve">PASS (CI 요구사항 실행 결과; 단계별 내역은 CI artifact 참조)</t>
         </is>
       </c>
     </row>
@@ -10796,7 +11732,7 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t xml:space="preserve">PASS</t>
+          <t xml:space="preserve">PASS (CI 요구사항 실행 결과; 단계별 내역은 CI artifact 참조)</t>
         </is>
       </c>
     </row>
@@ -10813,7 +11749,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t xml:space="preserve">PASS</t>
+          <t xml:space="preserve">PASS (CI 요구사항 실행 결과; 단계별 내역은 CI artifact 참조)</t>
         </is>
       </c>
     </row>
@@ -10830,7 +11766,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t xml:space="preserve">PASS</t>
+          <t xml:space="preserve">PASS (CI 요구사항 실행 결과; 단계별 내역은 CI artifact 참조)</t>
         </is>
       </c>
     </row>
@@ -10847,7 +11783,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t xml:space="preserve">PASS</t>
+          <t xml:space="preserve">PASS (CI 요구사항 실행 결과; 단계별 내역은 CI artifact 참조)</t>
         </is>
       </c>
     </row>
@@ -10864,7 +11800,7 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t xml:space="preserve">PASS</t>
+          <t xml:space="preserve">PASS (CI 요구사항 실행 결과; 단계별 내역은 CI artifact 참조)</t>
         </is>
       </c>
     </row>
@@ -10881,7 +11817,7 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t xml:space="preserve">PASS</t>
+          <t xml:space="preserve">PASS (CI 요구사항 실행 결과; 단계별 내역은 CI artifact 참조)</t>
         </is>
       </c>
     </row>
@@ -10898,7 +11834,7 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t xml:space="preserve">PASS</t>
+          <t xml:space="preserve">PASS (CI 요구사항 실행 결과; 단계별 내역은 CI artifact 참조)</t>
         </is>
       </c>
     </row>
@@ -10915,7 +11851,7 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t xml:space="preserve">PASS</t>
+          <t xml:space="preserve">PASS (CI 요구사항 실행 결과; 단계별 내역은 CI artifact 참조)</t>
         </is>
       </c>
     </row>
@@ -10932,7 +11868,7 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t xml:space="preserve">PASS</t>
+          <t xml:space="preserve">PASS (CI 요구사항 실행 결과; 단계별 내역은 CI artifact 참조)</t>
         </is>
       </c>
     </row>
@@ -10949,7 +11885,7 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t xml:space="preserve">PASS</t>
+          <t xml:space="preserve">PASS (CI 요구사항 실행 결과; 단계별 내역은 CI artifact 참조)</t>
         </is>
       </c>
     </row>
@@ -10966,7 +11902,7 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t xml:space="preserve">PASS</t>
+          <t xml:space="preserve">PASS (CI 요구사항 실행 결과; 단계별 내역은 CI artifact 참조)</t>
         </is>
       </c>
     </row>
@@ -10983,7 +11919,7 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t xml:space="preserve">PASS</t>
+          <t xml:space="preserve">PASS (CI 요구사항 실행 결과; 단계별 내역은 CI artifact 참조)</t>
         </is>
       </c>
     </row>
@@ -11000,7 +11936,7 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t xml:space="preserve">PASS</t>
+          <t xml:space="preserve">PASS (CI 요구사항 실행 결과; 단계별 내역은 CI artifact 참조)</t>
         </is>
       </c>
     </row>
@@ -11017,7 +11953,7 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t xml:space="preserve">PASS</t>
+          <t xml:space="preserve">PASS (CI 요구사항 실행 결과; 단계별 내역은 CI artifact 참조)</t>
         </is>
       </c>
     </row>
@@ -11034,7 +11970,7 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t xml:space="preserve">PASS</t>
+          <t xml:space="preserve">PASS (CI 요구사항 실행 결과; 단계별 내역은 CI artifact 참조)</t>
         </is>
       </c>
     </row>
@@ -11051,7 +11987,7 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t xml:space="preserve">PASS</t>
+          <t xml:space="preserve">PASS (CI 요구사항 실행 결과; 단계별 내역은 CI artifact 참조)</t>
         </is>
       </c>
     </row>
@@ -11068,7 +12004,7 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t xml:space="preserve">PASS</t>
+          <t xml:space="preserve">PASS (CI 요구사항 실행 결과; 단계별 내역은 CI artifact 참조)</t>
         </is>
       </c>
     </row>
@@ -11085,7 +12021,7 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t xml:space="preserve">PASS</t>
+          <t xml:space="preserve">PASS (CI 요구사항 실행 결과; 단계별 내역은 CI artifact 참조)</t>
         </is>
       </c>
     </row>
@@ -11102,7 +12038,7 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t xml:space="preserve">PASS</t>
+          <t xml:space="preserve">PASS (CI 요구사항 실행 결과; 단계별 내역은 CI artifact 참조)</t>
         </is>
       </c>
     </row>
@@ -11119,7 +12055,7 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t xml:space="preserve">PASS</t>
+          <t xml:space="preserve">PASS (CI 요구사항 실행 결과; 단계별 내역은 CI artifact 참조)</t>
         </is>
       </c>
     </row>
@@ -11136,7 +12072,7 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t xml:space="preserve">PASS</t>
+          <t xml:space="preserve">PASS (CI 요구사항 실행 결과; 단계별 내역은 CI artifact 참조)</t>
         </is>
       </c>
     </row>
@@ -11153,7 +12089,7 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t xml:space="preserve">PASS</t>
+          <t xml:space="preserve">PASS (CI 요구사항 실행 결과; 단계별 내역은 CI artifact 참조)</t>
         </is>
       </c>
     </row>
@@ -11170,7 +12106,7 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t xml:space="preserve">PASS</t>
+          <t xml:space="preserve">PASS (CI 요구사항 실행 결과; 단계별 내역은 CI artifact 참조)</t>
         </is>
       </c>
     </row>
@@ -11187,7 +12123,7 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t xml:space="preserve">PASS</t>
+          <t xml:space="preserve">PASS (CI 요구사항 실행 결과; 단계별 내역은 CI artifact 참조)</t>
         </is>
       </c>
     </row>
@@ -11204,7 +12140,7 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t xml:space="preserve">PASS</t>
+          <t xml:space="preserve">PASS (CI 요구사항 실행 결과; 단계별 내역은 CI artifact 참조)</t>
         </is>
       </c>
     </row>
@@ -11221,7 +12157,7 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t xml:space="preserve">PASS</t>
+          <t xml:space="preserve">PASS (CI 요구사항 실행 결과; 단계별 내역은 CI artifact 참조)</t>
         </is>
       </c>
     </row>
@@ -11238,7 +12174,7 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t xml:space="preserve">PASS</t>
+          <t xml:space="preserve">PASS (CI 요구사항 실행 결과; 단계별 내역은 CI artifact 참조)</t>
         </is>
       </c>
     </row>
@@ -11255,7 +12191,7 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t xml:space="preserve">PASS</t>
+          <t xml:space="preserve">PASS (CI 요구사항 실행 결과; 단계별 내역은 CI artifact 참조)</t>
         </is>
       </c>
     </row>
@@ -11272,7 +12208,7 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t xml:space="preserve">PASS</t>
+          <t xml:space="preserve">PASS (CI 요구사항 실행 결과; 단계별 내역은 CI artifact 참조)</t>
         </is>
       </c>
     </row>
@@ -11289,7 +12225,7 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t xml:space="preserve">PASS</t>
+          <t xml:space="preserve">PASS (CI 요구사항 실행 결과; 단계별 내역은 CI artifact 참조)</t>
         </is>
       </c>
     </row>
@@ -11306,7 +12242,7 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t xml:space="preserve">PASS</t>
+          <t xml:space="preserve">PASS (CI 요구사항 실행 결과; 단계별 내역은 CI artifact 참조)</t>
         </is>
       </c>
     </row>
@@ -11323,7 +12259,7 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t xml:space="preserve">PASS</t>
+          <t xml:space="preserve">PASS (CI 요구사항 실행 결과; 단계별 내역은 CI artifact 참조)</t>
         </is>
       </c>
     </row>
@@ -11340,7 +12276,7 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t xml:space="preserve">PASS</t>
+          <t xml:space="preserve">PASS (CI 요구사항 실행 결과; 단계별 내역은 CI artifact 참조)</t>
         </is>
       </c>
     </row>
@@ -11357,7 +12293,7 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t xml:space="preserve">PASS</t>
+          <t xml:space="preserve">PASS (CI 요구사항 실행 결과; 단계별 내역은 CI artifact 참조)</t>
         </is>
       </c>
     </row>
@@ -11374,7 +12310,7 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t xml:space="preserve">PASS</t>
+          <t xml:space="preserve">PASS (CI 요구사항 실행 결과; 단계별 내역은 CI artifact 참조)</t>
         </is>
       </c>
     </row>
@@ -11391,7 +12327,7 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t xml:space="preserve">PASS</t>
+          <t xml:space="preserve">PASS (CI 요구사항 실행 결과; 단계별 내역은 CI artifact 참조)</t>
         </is>
       </c>
     </row>
@@ -11408,7 +12344,7 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t xml:space="preserve">PASS</t>
+          <t xml:space="preserve">PASS (CI 요구사항 실행 결과; 단계별 내역은 CI artifact 참조)</t>
         </is>
       </c>
     </row>
@@ -11425,7 +12361,7 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t xml:space="preserve">PASS</t>
+          <t xml:space="preserve">PASS (CI 요구사항 실행 결과; 단계별 내역은 CI artifact 참조)</t>
         </is>
       </c>
     </row>
@@ -11442,7 +12378,7 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t xml:space="preserve">PASS</t>
+          <t xml:space="preserve">PASS (CI 요구사항 실행 결과; 단계별 내역은 CI artifact 참조)</t>
         </is>
       </c>
     </row>
@@ -11459,7 +12395,7 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t xml:space="preserve">PASS</t>
+          <t xml:space="preserve">PASS (CI 요구사항 실행 결과; 단계별 내역은 CI artifact 참조)</t>
         </is>
       </c>
     </row>
@@ -11476,7 +12412,7 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t xml:space="preserve">PASS</t>
+          <t xml:space="preserve">PASS (CI 요구사항 실행 결과; 단계별 내역은 CI artifact 참조)</t>
         </is>
       </c>
     </row>
@@ -11493,7 +12429,7 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t xml:space="preserve">PASS</t>
+          <t xml:space="preserve">PASS (CI 요구사항 실행 결과; 단계별 내역은 CI artifact 참조)</t>
         </is>
       </c>
     </row>
@@ -11510,7 +12446,7 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t xml:space="preserve">PASS</t>
+          <t xml:space="preserve">PASS (CI 요구사항 실행 결과; 단계별 내역은 CI artifact 참조)</t>
         </is>
       </c>
     </row>
@@ -11527,7 +12463,7 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t xml:space="preserve">PASS</t>
+          <t xml:space="preserve">PASS (CI 요구사항 실행 결과; 단계별 내역은 CI artifact 참조)</t>
         </is>
       </c>
     </row>
@@ -11544,7 +12480,7 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t xml:space="preserve">PASS</t>
+          <t xml:space="preserve">PASS (CI 요구사항 실행 결과; 단계별 내역은 CI artifact 참조)</t>
         </is>
       </c>
     </row>
@@ -11561,7 +12497,7 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t xml:space="preserve">PASS</t>
+          <t xml:space="preserve">PASS (CI 요구사항 실행 결과; 단계별 내역은 CI artifact 참조)</t>
         </is>
       </c>
     </row>
@@ -11578,7 +12514,7 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t xml:space="preserve">PASS</t>
+          <t xml:space="preserve">PASS (CI 요구사항 실행 결과; 단계별 내역은 CI artifact 참조)</t>
         </is>
       </c>
     </row>
@@ -11595,7 +12531,7 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t xml:space="preserve">PASS</t>
+          <t xml:space="preserve">PASS (CI 요구사항 실행 결과; 단계별 내역은 CI artifact 참조)</t>
         </is>
       </c>
     </row>
@@ -11612,7 +12548,7 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t xml:space="preserve">PASS</t>
+          <t xml:space="preserve">PASS (CI 요구사항 실행 결과; 단계별 내역은 CI artifact 참조)</t>
         </is>
       </c>
     </row>
@@ -11629,7 +12565,7 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t xml:space="preserve">PASS</t>
+          <t xml:space="preserve">PASS (CI 요구사항 실행 결과; 단계별 내역은 CI artifact 참조)</t>
         </is>
       </c>
     </row>
@@ -11646,7 +12582,7 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t xml:space="preserve">PASS</t>
+          <t xml:space="preserve">PASS (CI 요구사항 실행 결과; 단계별 내역은 CI artifact 참조)</t>
         </is>
       </c>
     </row>
@@ -11663,7 +12599,7 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t xml:space="preserve">PASS</t>
+          <t xml:space="preserve">PASS (CI 요구사항 실행 결과; 단계별 내역은 CI artifact 참조)</t>
         </is>
       </c>
     </row>
@@ -11680,7 +12616,7 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t xml:space="preserve">PASS</t>
+          <t xml:space="preserve">PASS (CI 요구사항 실행 결과; 단계별 내역은 CI artifact 참조)</t>
         </is>
       </c>
     </row>
@@ -11697,7 +12633,7 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t xml:space="preserve">PASS</t>
+          <t xml:space="preserve">PASS (CI 요구사항 실행 결과; 단계별 내역은 CI artifact 참조)</t>
         </is>
       </c>
     </row>
@@ -11714,7 +12650,7 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t xml:space="preserve">PASS</t>
+          <t xml:space="preserve">PASS (CI 요구사항 실행 결과; 단계별 내역은 CI artifact 참조)</t>
         </is>
       </c>
     </row>
@@ -11731,7 +12667,7 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t xml:space="preserve">PASS</t>
+          <t xml:space="preserve">PASS (CI 요구사항 실행 결과; 단계별 내역은 CI artifact 참조)</t>
         </is>
       </c>
     </row>
@@ -11748,7 +12684,7 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t xml:space="preserve">PASS</t>
+          <t xml:space="preserve">PASS (CI 요구사항 실행 결과; 단계별 내역은 CI artifact 참조)</t>
         </is>
       </c>
     </row>
@@ -11765,7 +12701,7 @@
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t xml:space="preserve">PASS</t>
+          <t xml:space="preserve">PASS (CI 요구사항 실행 결과; 단계별 내역은 CI artifact 참조)</t>
         </is>
       </c>
     </row>
@@ -11782,7 +12718,7 @@
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t xml:space="preserve">PASS</t>
+          <t xml:space="preserve">PASS (CI 요구사항 실행 결과; 단계별 내역은 CI artifact 참조)</t>
         </is>
       </c>
     </row>
@@ -11799,7 +12735,7 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t xml:space="preserve">PASS</t>
+          <t xml:space="preserve">PASS (CI 요구사항 실행 결과; 단계별 내역은 CI artifact 참조)</t>
         </is>
       </c>
     </row>
@@ -11816,7 +12752,7 @@
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t xml:space="preserve">PASS</t>
+          <t xml:space="preserve">PASS (CI 요구사항 실행 결과; 단계별 내역은 CI artifact 참조)</t>
         </is>
       </c>
     </row>
@@ -11833,7 +12769,7 @@
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t xml:space="preserve">PASS</t>
+          <t xml:space="preserve">PASS (CI 요구사항 실행 결과; 단계별 내역은 CI artifact 참조)</t>
         </is>
       </c>
     </row>
@@ -11850,7 +12786,7 @@
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t xml:space="preserve">PASS</t>
+          <t xml:space="preserve">PASS (CI 요구사항 실행 결과; 단계별 내역은 CI artifact 참조)</t>
         </is>
       </c>
     </row>
@@ -11867,7 +12803,7 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t xml:space="preserve">PASS</t>
+          <t xml:space="preserve">PASS (CI 요구사항 실행 결과; 단계별 내역은 CI artifact 참조)</t>
         </is>
       </c>
     </row>
@@ -11884,7 +12820,7 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t xml:space="preserve">PASS</t>
+          <t xml:space="preserve">PASS (CI 요구사항 실행 결과; 단계별 내역은 CI artifact 참조)</t>
         </is>
       </c>
     </row>
@@ -11901,7 +12837,7 @@
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t xml:space="preserve">PASS</t>
+          <t xml:space="preserve">PASS (CI 요구사항 실행 결과; 단계별 내역은 CI artifact 참조)</t>
         </is>
       </c>
     </row>
@@ -11918,7 +12854,7 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t xml:space="preserve">PASS</t>
+          <t xml:space="preserve">PASS (CI 요구사항 실행 결과; 단계별 내역은 CI artifact 참조)</t>
         </is>
       </c>
     </row>
@@ -11935,7 +12871,7 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t xml:space="preserve">PASS</t>
+          <t xml:space="preserve">PASS (CI 요구사항 실행 결과; 단계별 내역은 CI artifact 참조)</t>
         </is>
       </c>
     </row>
@@ -11952,7 +12888,7 @@
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t xml:space="preserve">PASS</t>
+          <t xml:space="preserve">PASS (CI 요구사항 실행 결과; 단계별 내역은 CI artifact 참조)</t>
         </is>
       </c>
     </row>
@@ -11969,7 +12905,7 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t xml:space="preserve">PASS</t>
+          <t xml:space="preserve">PASS (CI 요구사항 실행 결과; 단계별 내역은 CI artifact 참조)</t>
         </is>
       </c>
     </row>
@@ -11986,7 +12922,7 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t xml:space="preserve">PASS</t>
+          <t xml:space="preserve">PASS (CI 요구사항 실행 결과; 단계별 내역은 CI artifact 참조)</t>
         </is>
       </c>
     </row>
@@ -12003,7 +12939,7 @@
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t xml:space="preserve">PASS</t>
+          <t xml:space="preserve">PASS (CI 요구사항 실행 결과; 단계별 내역은 CI artifact 참조)</t>
         </is>
       </c>
     </row>
@@ -12020,7 +12956,7 @@
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t xml:space="preserve">PASS</t>
+          <t xml:space="preserve">PASS (CI 요구사항 실행 결과; 단계별 내역은 CI artifact 참조)</t>
         </is>
       </c>
     </row>
@@ -12037,7 +12973,7 @@
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t xml:space="preserve">PASS</t>
+          <t xml:space="preserve">PASS (CI 요구사항 실행 결과; 단계별 내역은 CI artifact 참조)</t>
         </is>
       </c>
     </row>
@@ -12054,7 +12990,7 @@
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t xml:space="preserve">PASS</t>
+          <t xml:space="preserve">PASS (CI 요구사항 실행 결과; 단계별 내역은 CI artifact 참조)</t>
         </is>
       </c>
     </row>
@@ -12071,7 +13007,7 @@
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t xml:space="preserve">PASS</t>
+          <t xml:space="preserve">PASS (CI 요구사항 실행 결과; 단계별 내역은 CI artifact 참조)</t>
         </is>
       </c>
     </row>
@@ -12088,7 +13024,7 @@
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t xml:space="preserve">PASS</t>
+          <t xml:space="preserve">PASS (CI 요구사항 실행 결과; 단계별 내역은 CI artifact 참조)</t>
         </is>
       </c>
     </row>
@@ -12105,7 +13041,7 @@
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t xml:space="preserve">PASS</t>
+          <t xml:space="preserve">PASS (CI 요구사항 실행 결과; 단계별 내역은 CI artifact 참조)</t>
         </is>
       </c>
     </row>
@@ -12122,7 +13058,7 @@
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t xml:space="preserve">PASS</t>
+          <t xml:space="preserve">PASS (CI 요구사항 실행 결과; 단계별 내역은 CI artifact 참조)</t>
         </is>
       </c>
     </row>
@@ -12139,7 +13075,7 @@
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t xml:space="preserve">PASS</t>
+          <t xml:space="preserve">PASS (CI 요구사항 실행 결과; 단계별 내역은 CI artifact 참조)</t>
         </is>
       </c>
     </row>
@@ -12156,7 +13092,7 @@
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t xml:space="preserve">PASS</t>
+          <t xml:space="preserve">PASS (CI 요구사항 실행 결과; 단계별 내역은 CI artifact 참조)</t>
         </is>
       </c>
     </row>
@@ -12173,7 +13109,7 @@
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t xml:space="preserve">PASS</t>
+          <t xml:space="preserve">PASS (CI 요구사항 실행 결과; 단계별 내역은 CI artifact 참조)</t>
         </is>
       </c>
     </row>
@@ -12190,7 +13126,7 @@
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t xml:space="preserve">PASS</t>
+          <t xml:space="preserve">PASS (CI 요구사항 실행 결과; 단계별 내역은 CI artifact 참조)</t>
         </is>
       </c>
     </row>
@@ -12207,7 +13143,7 @@
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t xml:space="preserve">PASS</t>
+          <t xml:space="preserve">PASS (CI 요구사항 실행 결과; 단계별 내역은 CI artifact 참조)</t>
         </is>
       </c>
     </row>
@@ -12224,7 +13160,7 @@
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t xml:space="preserve">PASS</t>
+          <t xml:space="preserve">PASS (CI 요구사항 실행 결과; 단계별 내역은 CI artifact 참조)</t>
         </is>
       </c>
     </row>
@@ -12241,7 +13177,7 @@
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t xml:space="preserve">PASS</t>
+          <t xml:space="preserve">PASS (CI 요구사항 실행 결과; 단계별 내역은 CI artifact 참조)</t>
         </is>
       </c>
     </row>
@@ -12258,7 +13194,7 @@
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t xml:space="preserve">PASS</t>
+          <t xml:space="preserve">PASS (CI 요구사항 실행 결과; 단계별 내역은 CI artifact 참조)</t>
         </is>
       </c>
     </row>
@@ -12275,7 +13211,7 @@
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t xml:space="preserve">PASS</t>
+          <t xml:space="preserve">PASS (CI 요구사항 실행 결과; 단계별 내역은 CI artifact 참조)</t>
         </is>
       </c>
     </row>
@@ -12292,7 +13228,7 @@
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t xml:space="preserve">PASS</t>
+          <t xml:space="preserve">PASS (CI 요구사항 실행 결과; 단계별 내역은 CI artifact 참조)</t>
         </is>
       </c>
     </row>
@@ -12309,7 +13245,7 @@
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t xml:space="preserve">PASS</t>
+          <t xml:space="preserve">PASS (CI 요구사항 실행 결과; 단계별 내역은 CI artifact 참조)</t>
         </is>
       </c>
     </row>
@@ -12326,7 +13262,7 @@
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t xml:space="preserve">PASS</t>
+          <t xml:space="preserve">PASS (CI 요구사항 실행 결과; 단계별 내역은 CI artifact 참조)</t>
         </is>
       </c>
     </row>
@@ -12343,7 +13279,7 @@
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t xml:space="preserve">PASS</t>
+          <t xml:space="preserve">PASS (CI 요구사항 실행 결과; 단계별 내역은 CI artifact 참조)</t>
         </is>
       </c>
     </row>
@@ -12360,7 +13296,7 @@
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t xml:space="preserve">PASS</t>
+          <t xml:space="preserve">PASS (CI 요구사항 실행 결과; 단계별 내역은 CI artifact 참조)</t>
         </is>
       </c>
     </row>
@@ -12377,7 +13313,7 @@
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t xml:space="preserve">PASS</t>
+          <t xml:space="preserve">PASS (CI 요구사항 실행 결과; 단계별 내역은 CI artifact 참조)</t>
         </is>
       </c>
     </row>
@@ -12394,7 +13330,7 @@
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t xml:space="preserve">PASS</t>
+          <t xml:space="preserve">PASS (CI 요구사항 실행 결과; 단계별 내역은 CI artifact 참조)</t>
         </is>
       </c>
     </row>
@@ -12411,7 +13347,7 @@
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t xml:space="preserve">PASS</t>
+          <t xml:space="preserve">PASS (CI 요구사항 실행 결과; 단계별 내역은 CI artifact 참조)</t>
         </is>
       </c>
     </row>
@@ -12428,7 +13364,7 @@
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t xml:space="preserve">PASS</t>
+          <t xml:space="preserve">PASS (CI 요구사항 실행 결과; 단계별 내역은 CI artifact 참조)</t>
         </is>
       </c>
     </row>
@@ -12445,7 +13381,7 @@
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t xml:space="preserve">PASS</t>
+          <t xml:space="preserve">PASS (CI 요구사항 실행 결과; 단계별 내역은 CI artifact 참조)</t>
         </is>
       </c>
     </row>
@@ -12462,7 +13398,7 @@
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t xml:space="preserve">PASS</t>
+          <t xml:space="preserve">PASS (CI 요구사항 실행 결과; 단계별 내역은 CI artifact 참조)</t>
         </is>
       </c>
     </row>
@@ -12479,7 +13415,7 @@
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t xml:space="preserve">PASS</t>
+          <t xml:space="preserve">PASS (CI 요구사항 실행 결과; 단계별 내역은 CI artifact 참조)</t>
         </is>
       </c>
     </row>
@@ -12496,7 +13432,7 @@
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t xml:space="preserve">PASS</t>
+          <t xml:space="preserve">PASS (CI 요구사항 실행 결과; 단계별 내역은 CI artifact 참조)</t>
         </is>
       </c>
     </row>
@@ -12513,7 +13449,7 @@
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t xml:space="preserve">PASS</t>
+          <t xml:space="preserve">PASS (CI 요구사항 실행 결과; 단계별 내역은 CI artifact 참조)</t>
         </is>
       </c>
     </row>
@@ -12530,7 +13466,7 @@
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t xml:space="preserve">PASS</t>
+          <t xml:space="preserve">PASS (CI 요구사항 실행 결과; 단계별 내역은 CI artifact 참조)</t>
         </is>
       </c>
     </row>
@@ -12547,7 +13483,7 @@
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t xml:space="preserve">PASS</t>
+          <t xml:space="preserve">PASS (CI 요구사항 실행 결과; 단계별 내역은 CI artifact 참조)</t>
         </is>
       </c>
     </row>
@@ -12564,7 +13500,7 @@
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t xml:space="preserve">PASS</t>
+          <t xml:space="preserve">PASS (CI 요구사항 실행 결과; 단계별 내역은 CI artifact 참조)</t>
         </is>
       </c>
     </row>
@@ -12581,7 +13517,7 @@
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t xml:space="preserve">PASS</t>
+          <t xml:space="preserve">PASS (CI 요구사항 실행 결과; 단계별 내역은 CI artifact 참조)</t>
         </is>
       </c>
     </row>
@@ -12598,7 +13534,7 @@
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t xml:space="preserve">PASS</t>
+          <t xml:space="preserve">PASS (CI 요구사항 실행 결과; 단계별 내역은 CI artifact 참조)</t>
         </is>
       </c>
     </row>
@@ -12615,7 +13551,7 @@
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t xml:space="preserve">PASS</t>
+          <t xml:space="preserve">PASS (CI 요구사항 실행 결과; 단계별 내역은 CI artifact 참조)</t>
         </is>
       </c>
     </row>
@@ -12632,7 +13568,7 @@
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t xml:space="preserve">PASS</t>
+          <t xml:space="preserve">PASS (CI 요구사항 실행 결과; 단계별 내역은 CI artifact 참조)</t>
         </is>
       </c>
     </row>
@@ -12649,7 +13585,7 @@
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t xml:space="preserve">PASS</t>
+          <t xml:space="preserve">PASS (CI 요구사항 실행 결과; 단계별 내역은 CI artifact 참조)</t>
         </is>
       </c>
     </row>
@@ -12666,7 +13602,7 @@
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t xml:space="preserve">PASS</t>
+          <t xml:space="preserve">PASS (CI 요구사항 실행 결과; 단계별 내역은 CI artifact 참조)</t>
         </is>
       </c>
     </row>
@@ -12683,7 +13619,7 @@
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t xml:space="preserve">PASS</t>
+          <t xml:space="preserve">PASS (CI 요구사항 실행 결과; 단계별 내역은 CI artifact 참조)</t>
         </is>
       </c>
     </row>
@@ -12700,7 +13636,7 @@
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t xml:space="preserve">PASS</t>
+          <t xml:space="preserve">PASS (CI 요구사항 실행 결과; 단계별 내역은 CI artifact 참조)</t>
         </is>
       </c>
     </row>
@@ -12717,7 +13653,7 @@
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t xml:space="preserve">PASS</t>
+          <t xml:space="preserve">PASS (CI 요구사항 실행 결과; 단계별 내역은 CI artifact 참조)</t>
         </is>
       </c>
     </row>
@@ -12734,7 +13670,7 @@
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t xml:space="preserve">PASS</t>
+          <t xml:space="preserve">PASS (CI 요구사항 실행 결과; 단계별 내역은 CI artifact 참조)</t>
         </is>
       </c>
     </row>
@@ -12751,7 +13687,7 @@
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t xml:space="preserve">PASS</t>
+          <t xml:space="preserve">PASS (CI 요구사항 실행 결과; 단계별 내역은 CI artifact 참조)</t>
         </is>
       </c>
     </row>
@@ -12768,7 +13704,7 @@
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t xml:space="preserve">PASS</t>
+          <t xml:space="preserve">PASS (CI 요구사항 실행 결과; 단계별 내역은 CI artifact 참조)</t>
         </is>
       </c>
     </row>
@@ -12785,7 +13721,7 @@
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t xml:space="preserve">PASS</t>
+          <t xml:space="preserve">PASS (CI 요구사항 실행 결과; 단계별 내역은 CI artifact 참조)</t>
         </is>
       </c>
     </row>
@@ -12802,7 +13738,7 @@
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t xml:space="preserve">PASS</t>
+          <t xml:space="preserve">PASS (CI 요구사항 실행 결과; 단계별 내역은 CI artifact 참조)</t>
         </is>
       </c>
     </row>
@@ -12819,7 +13755,7 @@
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t xml:space="preserve">PASS</t>
+          <t xml:space="preserve">PASS (CI 요구사항 실행 결과; 단계별 내역은 CI artifact 참조)</t>
         </is>
       </c>
     </row>
@@ -12836,7 +13772,7 @@
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t xml:space="preserve">PASS</t>
+          <t xml:space="preserve">PASS (CI 요구사항 실행 결과; 단계별 내역은 CI artifact 참조)</t>
         </is>
       </c>
     </row>
@@ -12853,7 +13789,7 @@
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t xml:space="preserve">PASS</t>
+          <t xml:space="preserve">PASS (CI 요구사항 실행 결과; 단계별 내역은 CI artifact 참조)</t>
         </is>
       </c>
     </row>
@@ -12870,7 +13806,7 @@
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t xml:space="preserve">PASS</t>
+          <t xml:space="preserve">PASS (CI 요구사항 실행 결과; 단계별 내역은 CI artifact 참조)</t>
         </is>
       </c>
     </row>
@@ -12887,7 +13823,7 @@
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t xml:space="preserve">PASS</t>
+          <t xml:space="preserve">PASS (CI 요구사항 실행 결과; 단계별 내역은 CI artifact 참조)</t>
         </is>
       </c>
     </row>
@@ -12904,7 +13840,7 @@
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t xml:space="preserve">PASS</t>
+          <t xml:space="preserve">PASS (CI 요구사항 실행 결과; 단계별 내역은 CI artifact 참조)</t>
         </is>
       </c>
     </row>
@@ -12921,7 +13857,7 @@
       </c>
       <c r="C157" t="inlineStr">
         <is>
-          <t xml:space="preserve">PASS</t>
+          <t xml:space="preserve">PASS (CI 요구사항 실행 결과; 단계별 내역은 CI artifact 참조)</t>
         </is>
       </c>
     </row>
@@ -12938,7 +13874,7 @@
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t xml:space="preserve">PASS</t>
+          <t xml:space="preserve">PASS (CI 요구사항 실행 결과; 단계별 내역은 CI artifact 참조)</t>
         </is>
       </c>
     </row>
@@ -12955,7 +13891,7 @@
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t xml:space="preserve">PASS</t>
+          <t xml:space="preserve">PASS (CI 요구사항 실행 결과; 단계별 내역은 CI artifact 참조)</t>
         </is>
       </c>
     </row>
@@ -12972,7 +13908,7 @@
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t xml:space="preserve">PASS</t>
+          <t xml:space="preserve">PASS (CI 요구사항 실행 결과; 단계별 내역은 CI artifact 참조)</t>
         </is>
       </c>
     </row>
@@ -12989,7 +13925,7 @@
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t xml:space="preserve">PASS</t>
+          <t xml:space="preserve">PASS (CI 요구사항 실행 결과; 단계별 내역은 CI artifact 참조)</t>
         </is>
       </c>
     </row>
@@ -13006,7 +13942,7 @@
       </c>
       <c r="C162" t="inlineStr">
         <is>
-          <t xml:space="preserve">PASS</t>
+          <t xml:space="preserve">PASS (CI 요구사항 실행 결과; 단계별 내역은 CI artifact 참조)</t>
         </is>
       </c>
     </row>
@@ -13023,7 +13959,7 @@
       </c>
       <c r="C163" t="inlineStr">
         <is>
-          <t xml:space="preserve">PASS</t>
+          <t xml:space="preserve">PASS (CI 요구사항 실행 결과; 단계별 내역은 CI artifact 참조)</t>
         </is>
       </c>
     </row>
@@ -13040,7 +13976,7 @@
       </c>
       <c r="C164" t="inlineStr">
         <is>
-          <t xml:space="preserve">PASS</t>
+          <t xml:space="preserve">PASS (CI 요구사항 실행 결과; 단계별 내역은 CI artifact 참조)</t>
         </is>
       </c>
     </row>
@@ -13057,7 +13993,7 @@
       </c>
       <c r="C165" t="inlineStr">
         <is>
-          <t xml:space="preserve">PASS</t>
+          <t xml:space="preserve">PASS (CI 요구사항 실행 결과; 단계별 내역은 CI artifact 참조)</t>
         </is>
       </c>
     </row>
@@ -13074,7 +14010,7 @@
       </c>
       <c r="C166" t="inlineStr">
         <is>
-          <t xml:space="preserve">PASS</t>
+          <t xml:space="preserve">PASS (CI 요구사항 실행 결과; 단계별 내역은 CI artifact 참조)</t>
         </is>
       </c>
     </row>
@@ -13091,7 +14027,7 @@
       </c>
       <c r="C167" t="inlineStr">
         <is>
-          <t xml:space="preserve">PASS</t>
+          <t xml:space="preserve">PASS (CI 요구사항 실행 결과; 단계별 내역은 CI artifact 참조)</t>
         </is>
       </c>
     </row>
@@ -13108,7 +14044,7 @@
       </c>
       <c r="C168" t="inlineStr">
         <is>
-          <t xml:space="preserve">PASS</t>
+          <t xml:space="preserve">PASS (CI 요구사항 실행 결과; 단계별 내역은 CI artifact 참조)</t>
         </is>
       </c>
     </row>
@@ -13125,7 +14061,7 @@
       </c>
       <c r="C169" t="inlineStr">
         <is>
-          <t xml:space="preserve">PASS</t>
+          <t xml:space="preserve">PASS (CI 요구사항 실행 결과; 단계별 내역은 CI artifact 참조)</t>
         </is>
       </c>
     </row>
@@ -13142,7 +14078,7 @@
       </c>
       <c r="C170" t="inlineStr">
         <is>
-          <t xml:space="preserve">PASS</t>
+          <t xml:space="preserve">PASS (CI 요구사항 실행 결과; 단계별 내역은 CI artifact 참조)</t>
         </is>
       </c>
     </row>
@@ -13159,7 +14095,7 @@
       </c>
       <c r="C171" t="inlineStr">
         <is>
-          <t xml:space="preserve">PASS</t>
+          <t xml:space="preserve">PASS (CI 요구사항 실행 결과; 단계별 내역은 CI artifact 참조)</t>
         </is>
       </c>
     </row>
@@ -13176,7 +14112,7 @@
       </c>
       <c r="C172" t="inlineStr">
         <is>
-          <t xml:space="preserve">PASS</t>
+          <t xml:space="preserve">PASS (CI 요구사항 실행 결과; 단계별 내역은 CI artifact 참조)</t>
         </is>
       </c>
     </row>
@@ -13193,7 +14129,7 @@
       </c>
       <c r="C173" t="inlineStr">
         <is>
-          <t xml:space="preserve">PASS</t>
+          <t xml:space="preserve">PASS (CI 요구사항 실행 결과; 단계별 내역은 CI artifact 참조)</t>
         </is>
       </c>
     </row>
@@ -13210,7 +14146,7 @@
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t xml:space="preserve">PASS</t>
+          <t xml:space="preserve">PASS (CI 요구사항 실행 결과; 단계별 내역은 CI artifact 참조)</t>
         </is>
       </c>
     </row>
@@ -13227,7 +14163,7 @@
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t xml:space="preserve">PASS</t>
+          <t xml:space="preserve">PASS (CI 요구사항 실행 결과; 단계별 내역은 CI artifact 참조)</t>
         </is>
       </c>
     </row>
@@ -13244,7 +14180,7 @@
       </c>
       <c r="C176" t="inlineStr">
         <is>
-          <t xml:space="preserve">PASS</t>
+          <t xml:space="preserve">PASS (CI 요구사항 실행 결과; 단계별 내역은 CI artifact 참조)</t>
         </is>
       </c>
     </row>
@@ -13261,7 +14197,7 @@
       </c>
       <c r="C177" t="inlineStr">
         <is>
-          <t xml:space="preserve">PASS</t>
+          <t xml:space="preserve">PASS (CI 요구사항 실행 결과; 단계별 내역은 CI artifact 참조)</t>
         </is>
       </c>
     </row>
@@ -13278,7 +14214,7 @@
       </c>
       <c r="C178" t="inlineStr">
         <is>
-          <t xml:space="preserve">PASS</t>
+          <t xml:space="preserve">PASS (CI 요구사항 실행 결과; 단계별 내역은 CI artifact 참조)</t>
         </is>
       </c>
     </row>
@@ -13295,7 +14231,7 @@
       </c>
       <c r="C179" t="inlineStr">
         <is>
-          <t xml:space="preserve">PASS</t>
+          <t xml:space="preserve">PASS (CI 요구사항 실행 결과; 단계별 내역은 CI artifact 참조)</t>
         </is>
       </c>
     </row>
@@ -13312,7 +14248,7 @@
       </c>
       <c r="C180" t="inlineStr">
         <is>
-          <t xml:space="preserve">PASS</t>
+          <t xml:space="preserve">PASS (CI 요구사항 실행 결과; 단계별 내역은 CI artifact 참조)</t>
         </is>
       </c>
     </row>
@@ -13329,7 +14265,7 @@
       </c>
       <c r="C181" t="inlineStr">
         <is>
-          <t xml:space="preserve">PASS</t>
+          <t xml:space="preserve">PASS (CI 요구사항 실행 결과; 단계별 내역은 CI artifact 참조)</t>
         </is>
       </c>
     </row>
@@ -13346,7 +14282,7 @@
       </c>
       <c r="C182" t="inlineStr">
         <is>
-          <t xml:space="preserve">PASS</t>
+          <t xml:space="preserve">PASS (CI 요구사항 실행 결과; 단계별 내역은 CI artifact 참조)</t>
         </is>
       </c>
     </row>
@@ -13363,7 +14299,7 @@
       </c>
       <c r="C183" t="inlineStr">
         <is>
-          <t xml:space="preserve">PASS</t>
+          <t xml:space="preserve">PASS (CI 요구사항 실행 결과; 단계별 내역은 CI artifact 참조)</t>
         </is>
       </c>
     </row>
@@ -13380,7 +14316,7 @@
       </c>
       <c r="C184" t="inlineStr">
         <is>
-          <t xml:space="preserve">PASS</t>
+          <t xml:space="preserve">PASS (CI 요구사항 실행 결과; 단계별 내역은 CI artifact 참조)</t>
         </is>
       </c>
     </row>
@@ -13397,7 +14333,7 @@
       </c>
       <c r="C185" t="inlineStr">
         <is>
-          <t xml:space="preserve">PASS</t>
+          <t xml:space="preserve">PASS (CI 요구사항 실행 결과; 단계별 내역은 CI artifact 참조)</t>
         </is>
       </c>
     </row>
@@ -13414,7 +14350,7 @@
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t xml:space="preserve">PASS</t>
+          <t xml:space="preserve">PASS (CI 요구사항 실행 결과; 단계별 내역은 CI artifact 참조)</t>
         </is>
       </c>
     </row>
@@ -13431,7 +14367,7 @@
       </c>
       <c r="C187" t="inlineStr">
         <is>
-          <t xml:space="preserve">PASS</t>
+          <t xml:space="preserve">PASS (CI 요구사항 실행 결과; 단계별 내역은 CI artifact 참조)</t>
         </is>
       </c>
     </row>
@@ -13448,7 +14384,7 @@
       </c>
       <c r="C188" t="inlineStr">
         <is>
-          <t xml:space="preserve">PASS</t>
+          <t xml:space="preserve">PASS (CI 요구사항 실행 결과; 단계별 내역은 CI artifact 참조)</t>
         </is>
       </c>
     </row>
@@ -13465,7 +14401,7 @@
       </c>
       <c r="C189" t="inlineStr">
         <is>
-          <t xml:space="preserve">PASS</t>
+          <t xml:space="preserve">PASS (CI 요구사항 실행 결과; 단계별 내역은 CI artifact 참조)</t>
         </is>
       </c>
     </row>
@@ -13482,11 +14418,385 @@
       </c>
       <c r="C190" t="inlineStr">
         <is>
-          <t xml:space="preserve">PASS</t>
+          <t xml:space="preserve">PASS (CI 요구사항 실행 결과; 단계별 내역은 CI artifact 참조)</t>
+        </is>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" t="inlineStr">
+        <is>
+          <t xml:space="preserve">190</t>
+        </is>
+      </c>
+      <c r="B191" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tests/test_quality_lifecycle.py::test_full_review_covers_train_and_eval</t>
+        </is>
+      </c>
+      <c r="C191" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PASS (CI 요구사항 실행 결과; 단계별 내역은 CI artifact 참조)</t>
+        </is>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" t="inlineStr">
+        <is>
+          <t xml:space="preserve">191</t>
+        </is>
+      </c>
+      <c r="B192" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tests/test_quality_lifecycle.py::test_full_review_rejects_or_fails_closed[reject]</t>
+        </is>
+      </c>
+      <c r="C192" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PASS (CI 요구사항 실행 결과; 단계별 내역은 CI artifact 참조)</t>
+        </is>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" t="inlineStr">
+        <is>
+          <t xml:space="preserve">192</t>
+        </is>
+      </c>
+      <c r="B193" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tests/test_quality_lifecycle.py::test_full_review_rejects_or_fails_closed[risk]</t>
+        </is>
+      </c>
+      <c r="C193" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PASS (CI 요구사항 실행 결과; 단계별 내역은 CI artifact 참조)</t>
+        </is>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" t="inlineStr">
+        <is>
+          <t xml:space="preserve">193</t>
+        </is>
+      </c>
+      <c r="B194" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tests/test_quality_lifecycle.py::test_full_review_rejects_or_fails_closed[broken]</t>
+        </is>
+      </c>
+      <c r="C194" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PASS (CI 요구사항 실행 결과; 단계별 내역은 CI artifact 참조)</t>
+        </is>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" t="inlineStr">
+        <is>
+          <t xml:space="preserve">194</t>
+        </is>
+      </c>
+      <c r="B195" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tests/test_quality_lifecycle.py::test_full_review_rejects_or_fails_closed[simulated]</t>
+        </is>
+      </c>
+      <c r="C195" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PASS (CI 요구사항 실행 결과; 단계별 내역은 CI artifact 참조)</t>
+        </is>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" t="inlineStr">
+        <is>
+          <t xml:space="preserve">195</t>
+        </is>
+      </c>
+      <c r="B196" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tests/test_quality_lifecycle.py::test_full_review_rejects_or_fails_closed[model_change]</t>
+        </is>
+      </c>
+      <c r="C196" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PASS (CI 요구사항 실행 결과; 단계별 내역은 CI artifact 참조)</t>
+        </is>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" t="inlineStr">
+        <is>
+          <t xml:space="preserve">196</t>
+        </is>
+      </c>
+      <c r="B197" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tests/test_quality_lifecycle.py::test_review_error_does_not_store_partial_pass</t>
+        </is>
+      </c>
+      <c r="C197" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PASS (CI 요구사항 실행 결과; 단계별 내역은 CI artifact 참조)</t>
+        </is>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" t="inlineStr">
+        <is>
+          <t xml:space="preserve">197</t>
+        </is>
+      </c>
+      <c r="B198" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tests/test_quality_lifecycle.py::test_old_preview_cannot_approve</t>
+        </is>
+      </c>
+      <c r="C198" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PASS (CI 요구사항 실행 결과; 단계별 내역은 CI artifact 참조)</t>
+        </is>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" t="inlineStr">
+        <is>
+          <t xml:space="preserve">198</t>
+        </is>
+      </c>
+      <c r="B199" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tests/test_quality_lifecycle.py::test_benchmark_registration_and_immutable_plan</t>
+        </is>
+      </c>
+      <c r="C199" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PASS (CI 요구사항 실행 결과; 단계별 내역은 CI artifact 참조)</t>
+        </is>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" t="inlineStr">
+        <is>
+          <t xml:space="preserve">199</t>
+        </is>
+      </c>
+      <c r="B200" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tests/test_quality_lifecycle.py::test_benchmark_limits_and_duplicates[cases0]</t>
+        </is>
+      </c>
+      <c r="C200" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PASS (CI 요구사항 실행 결과; 단계별 내역은 CI artifact 참조)</t>
+        </is>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" t="inlineStr">
+        <is>
+          <t xml:space="preserve">200</t>
+        </is>
+      </c>
+      <c r="B201" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tests/test_quality_lifecycle.py::test_benchmark_limits_and_duplicates[cases1]</t>
+        </is>
+      </c>
+      <c r="C201" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PASS (CI 요구사항 실행 결과; 단계별 내역은 CI artifact 참조)</t>
+        </is>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" t="inlineStr">
+        <is>
+          <t xml:space="preserve">201</t>
+        </is>
+      </c>
+      <c r="B202" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tests/test_quality_lifecycle.py::test_benchmark_limits_and_duplicates[cases2]</t>
+        </is>
+      </c>
+      <c r="C202" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PASS (CI 요구사항 실행 결과; 단계별 내역은 CI artifact 참조)</t>
+        </is>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" t="inlineStr">
+        <is>
+          <t xml:space="preserve">202</t>
+        </is>
+      </c>
+      <c r="B203" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tests/test_quality_lifecycle.py::test_benchmark_leakage_and_unknown_suite</t>
+        </is>
+      </c>
+      <c r="C203" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PASS (CI 요구사항 실행 결과; 단계별 내역은 CI artifact 참조)</t>
+        </is>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" t="inlineStr">
+        <is>
+          <t xml:space="preserve">203</t>
+        </is>
+      </c>
+      <c r="B204" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tests/test_quality_lifecycle.py::test_benchmark_exact_match_and_response_validation</t>
+        </is>
+      </c>
+      <c r="C204" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PASS (CI 요구사항 실행 결과; 단계별 내역은 CI artifact 참조)</t>
+        </is>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" t="inlineStr">
+        <is>
+          <t xml:space="preserve">204</t>
+        </is>
+      </c>
+      <c r="B205" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tests/test_quality_lifecycle.py::test_dashboard_no_worker_or_percent_claim</t>
+        </is>
+      </c>
+      <c r="C205" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PASS (CI 요구사항 실행 결과; 단계별 내역은 CI artifact 참조)</t>
+        </is>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" t="inlineStr">
+        <is>
+          <t xml:space="preserve">205</t>
+        </is>
+      </c>
+      <c r="B206" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tests/test_quality_lifecycle.py::test_candidate_selection_rollback_and_cas</t>
+        </is>
+      </c>
+      <c r="C206" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PASS (CI 요구사항 실행 결과; 단계별 내역은 CI artifact 참조)</t>
+        </is>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" t="inlineStr">
+        <is>
+          <t xml:space="preserve">206</t>
+        </is>
+      </c>
+      <c r="B207" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tests/test_quality_lifecycle.py::test_candidate_validation_blocks_bad_versions[tamper]</t>
+        </is>
+      </c>
+      <c r="C207" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PASS (CI 요구사항 실행 결과; 단계별 내역은 CI artifact 참조)</t>
+        </is>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" t="inlineStr">
+        <is>
+          <t xml:space="preserve">207</t>
+        </is>
+      </c>
+      <c r="B208" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tests/test_quality_lifecycle.py::test_candidate_validation_blocks_bad_versions[regression]</t>
+        </is>
+      </c>
+      <c r="C208" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PASS (CI 요구사항 실행 결과; 단계별 내역은 CI artifact 참조)</t>
+        </is>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" t="inlineStr">
+        <is>
+          <t xml:space="preserve">208</t>
+        </is>
+      </c>
+      <c r="B209" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tests/test_quality_lifecycle.py::test_candidate_validation_blocks_bad_versions[missing_benchmark]</t>
+        </is>
+      </c>
+      <c r="C209" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PASS (CI 요구사항 실행 결과; 단계별 내역은 CI artifact 참조)</t>
+        </is>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" t="inlineStr">
+        <is>
+          <t xml:space="preserve">209</t>
+        </is>
+      </c>
+      <c r="B210" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tests/test_quality_lifecycle.py::test_candidate_validation_blocks_bad_versions[fake]</t>
+        </is>
+      </c>
+      <c r="C210" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PASS (CI 요구사항 실행 결과; 단계별 내역은 CI artifact 참조)</t>
+        </is>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" t="inlineStr">
+        <is>
+          <t xml:space="preserve">210</t>
+        </is>
+      </c>
+      <c r="B211" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tests/test_quality_lifecycle.py::test_rollback_revalidates_previous_files</t>
+        </is>
+      </c>
+      <c r="C211" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PASS (CI 요구사항 실행 결과; 단계별 내역은 CI artifact 참조)</t>
+        </is>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" t="inlineStr">
+        <is>
+          <t xml:space="preserve">211</t>
+        </is>
+      </c>
+      <c r="B212" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tests/test_quality_lifecycle.py::test_lifecycle_owner_and_csrf</t>
+        </is>
+      </c>
+      <c r="C212" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PASS (CI 요구사항 실행 결과; 단계별 내역은 CI artifact 참조)</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:C190"/>
+  <autoFilter ref="A1:C212"/>
 </worksheet>
 </file>
</xml_diff>